<commit_message>
Session 2026-09-04: WO-P000-E20.001 lessons_audit built+rolled out, LM Studio VRAM-contention fix, peh-handoff v1.11. Also includes accumulated P_010/P_115/P_300/P_400/P_800/P_820/trading_journal work left uncommitted since 2026-09-02, not individually reviewed this session.
</commit_message>
<xml_diff>
--- a/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (QQQ)_v3.xlsx
+++ b/projects/P_010_Current_Market_Posture/data/excel_exports/History Grid (QQQ)_v3.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="27">
   <si>
     <t>High
 Price</t>
@@ -67,11 +67,11 @@
 Price</t>
   </si>
   <si>
+    <t>Medium</t>
+  </si>
+  <si>
     <t>Low
 Price</t>
-  </si>
-  <si>
-    <t>Triple Cross Medium</t>
   </si>
   <si>
     <t>Long
@@ -81,6 +81,9 @@
   <si>
     <t>Close
 Price</t>
+  </si>
+  <si>
+    <t>Long</t>
   </si>
   <si>
     <t>Predicted
@@ -93,6 +96,9 @@
 Difference</t>
   </si>
   <si>
+    <t>Short</t>
+  </si>
+  <si>
     <t>Volume</t>
   </si>
   <si>
@@ -102,17 +108,11 @@
     <t>ROC%</t>
   </si>
   <si>
-    <t>Triple Cross Short</t>
-  </si>
-  <si>
     <t>Williams
 EMAI</t>
   </si>
   <si>
     <t>Neural Index</t>
-  </si>
-  <si>
-    <t>Triple Cross Long</t>
   </si>
 </sst>
 </file>
@@ -150,10 +150,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" relativeIndent="0" readingOrder="0"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -466,9 +466,9 @@
     <col min="14" max="14" width="15.85546875" customWidth="1"/>
     <col min="15" max="15" width="12.85546875" customWidth="1"/>
     <col min="16" max="16" width="17.7109375" customWidth="1"/>
-    <col min="17" max="17" width="23.7109375" customWidth="1"/>
-    <col min="18" max="18" width="27" customWidth="1"/>
-    <col min="19" max="19" width="23.28515625" customWidth="1"/>
+    <col min="17" max="17" width="10" customWidth="1"/>
+    <col min="18" max="18" width="13.28515625" customWidth="1"/>
+    <col min="19" max="19" width="9.7109375" customWidth="1"/>
     <col min="20" max="22" width="14.5703125" customWidth="1"/>
     <col min="23" max="16384" width="8.7265625"/>
   </cols>
@@ -477,74 +477,74 @@
       <c r="A1" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="K1" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>25</v>
       </c>
       <c r="M1" t="s">
         <v>9</v>
       </c>
       <c r="O1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q1" t="s">
         <v>3</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="L2" s="2"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="L2" s="1"/>
       <c r="M2" t="s">
         <v>4</v>
       </c>
       <c r="N2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="O2" t="s">
         <v>10</v>
@@ -553,2940 +553,3076 @@
         <v>8</v>
       </c>
       <c r="Q2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="R2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S2" t="s">
-        <v>26</v>
-      </c>
-      <c r="T2" s="2"/>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
+        <v>18</v>
+      </c>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="1">
-        <v>46261</v>
+      <c r="A3" s="2">
+        <v>46269</v>
       </c>
       <c r="B3">
-        <v>4.66131591796875</v>
+        <v>3.72772216796875</v>
       </c>
       <c r="C3">
-        <v>-1.491943359375</v>
+        <v>2.60296630859375</v>
       </c>
       <c r="D3">
-        <v>-3.8359375</v>
+        <v>0.3096923828125</v>
       </c>
       <c r="E3">
-        <v>716.929992675781</v>
+        <v>719.344970703125</v>
       </c>
       <c r="F3">
-        <v>721.349975585938</v>
+        <v>721.859985351563</v>
       </c>
       <c r="G3">
-        <v>714.525024414063</v>
+        <v>716.559997558594</v>
       </c>
       <c r="H3">
-        <v>721.109985351563</v>
+        <v>718.960021972656</v>
       </c>
       <c r="I3">
-        <v>722.337341308594</v>
+        <v>722.363159179688</v>
       </c>
       <c r="J3">
-        <v>717.721252441406</v>
+        <v>716.705444335938</v>
       </c>
       <c r="K3">
-        <v>28723400</v>
+        <v>32780670</v>
       </c>
       <c r="L3">
-        <v>0.713811993598938</v>
+        <v>-0.234040766954422</v>
       </c>
       <c r="M3">
-        <v>74.1502151489258</v>
+        <v>47.793140411377</v>
       </c>
       <c r="N3">
-        <v>-12.5261697769165</v>
+        <v>-7.73266696929932</v>
       </c>
       <c r="O3" t="s">
         <v>1</v>
       </c>
       <c r="P3">
-        <v>35.1892890930176</v>
+        <v>57.7196006774902</v>
       </c>
       <c r="Q3">
-        <v>715.721313476563</v>
+        <v>716.620361328125</v>
       </c>
       <c r="R3">
-        <v>715.231018066406</v>
+        <v>715.381286621094</v>
       </c>
       <c r="S3">
-        <v>714.299743652344</v>
+        <v>714.463317871094</v>
       </c>
       <c r="T3">
-        <v>0.98736572265625</v>
+        <v>0.503173828125</v>
       </c>
       <c r="U3">
-        <v>3.19622802734375</v>
+        <v>0.14544677734375</v>
       </c>
       <c r="V3">
-        <v>4.6160888671875</v>
+        <v>5.65771484375</v>
       </c>
     </row>
     <row r="4" ht="19.5" customHeight="1">
-      <c r="A4" s="1">
-        <v>46260</v>
+      <c r="A4" s="2">
+        <v>46268</v>
       </c>
       <c r="B4">
-        <v>0.4306640625</v>
+        <v>1.111083984375</v>
       </c>
       <c r="C4">
-        <v>-6.2967529296875</v>
+        <v>0.99615478515625</v>
       </c>
       <c r="D4">
-        <v>-6.01812744140625</v>
+        <v>-2.15606689453125</v>
       </c>
       <c r="E4">
-        <v>708.409973144531</v>
+        <v>710.849975585938</v>
       </c>
       <c r="F4">
-        <v>713.02001953125</v>
+        <v>718.914978027344</v>
       </c>
       <c r="G4">
-        <v>707.969970703125</v>
+        <v>709.690002441406</v>
       </c>
       <c r="H4">
-        <v>711.369995117188</v>
+        <v>717.669982910156</v>
       </c>
       <c r="I4">
-        <v>714.13525390625</v>
+        <v>719.351440429688</v>
       </c>
       <c r="J4">
-        <v>708.566284179688</v>
+        <v>714.108703613281</v>
       </c>
       <c r="K4">
-        <v>20392300</v>
+        <v>29449700</v>
       </c>
       <c r="L4">
-        <v>-0.141427174210548</v>
+        <v>-0.0333281010389328</v>
       </c>
       <c r="M4">
-        <v>84.7684555053711</v>
+        <v>51.7985496520996</v>
       </c>
       <c r="N4">
-        <v>1.23760998249054</v>
+        <v>-23.523889541626</v>
       </c>
       <c r="O4" t="s">
         <v>1</v>
       </c>
       <c r="P4">
+        <v>50.7881851196289</v>
+      </c>
+      <c r="Q4">
+        <v>713.895751953125</v>
+      </c>
+      <c r="R4">
+        <v>714.236145019531</v>
+      </c>
+      <c r="S4">
+        <v>713.808471679688</v>
+      </c>
+      <c r="T4">
+        <v>0.43646240234375</v>
+      </c>
+      <c r="U4">
+        <v>4.418701171875</v>
+      </c>
+      <c r="V4">
+        <v>5.24273681640625</v>
+      </c>
+    </row>
+    <row r="5" ht="19.5" customHeight="1">
+      <c r="A5" s="2">
+        <v>46267</v>
+      </c>
+      <c r="B5">
+        <v>-4.34771728515625</v>
+      </c>
+      <c r="C5">
+        <v>-0.8651123046875</v>
+      </c>
+      <c r="D5">
+        <v>-4.5257568359375</v>
+      </c>
+      <c r="E5">
+        <v>707.099975585938</v>
+      </c>
+      <c r="F5">
+        <v>709.798889160156</v>
+      </c>
+      <c r="G5">
+        <v>705.099975585938</v>
+      </c>
+      <c r="H5">
+        <v>709.239990234375</v>
+      </c>
+      <c r="I5">
+        <v>712.845642089844</v>
+      </c>
+      <c r="J5">
+        <v>706.473327636719</v>
+      </c>
+      <c r="K5">
+        <v>23476200</v>
+      </c>
+      <c r="L5">
+        <v>-0.784281432628632</v>
+      </c>
+      <c r="M5">
+        <v>67.7316741943359</v>
+      </c>
+      <c r="N5">
+        <v>-9.31163692474365</v>
+      </c>
+      <c r="O5" t="s">
+        <v>23</v>
+      </c>
+      <c r="P5">
+        <v>-10.4177856445313</v>
+      </c>
+      <c r="Q5">
+        <v>710.752807617188</v>
+      </c>
+      <c r="R5">
+        <v>713.091125488281</v>
+      </c>
+      <c r="S5">
+        <v>713.333984375</v>
+      </c>
+      <c r="T5">
+        <v>3.0467529296875</v>
+      </c>
+      <c r="U5">
+        <v>1.37335205078125</v>
+      </c>
+      <c r="V5">
+        <v>6.372314453125</v>
+      </c>
+    </row>
+    <row r="6" ht="19.5" customHeight="1">
+      <c r="A6" s="2">
+        <v>46266</v>
+      </c>
+      <c r="B6">
+        <v>-4.03338623046875</v>
+      </c>
+      <c r="C6">
+        <v>-0.24066162109375</v>
+      </c>
+      <c r="D6">
+        <v>-4.17218017578125</v>
+      </c>
+      <c r="E6">
+        <v>707.390014648438</v>
+      </c>
+      <c r="F6">
+        <v>712.299987792969</v>
+      </c>
+      <c r="G6">
+        <v>704.659973144531</v>
+      </c>
+      <c r="H6">
+        <v>707.640014648438</v>
+      </c>
+      <c r="I6">
+        <v>711.4423828125</v>
+      </c>
+      <c r="J6">
+        <v>703.673706054688</v>
+      </c>
+      <c r="K6">
+        <v>35236100</v>
+      </c>
+      <c r="L6">
+        <v>-0.139043897390366</v>
+      </c>
+      <c r="M6">
+        <v>74.6861801147461</v>
+      </c>
+      <c r="N6">
+        <v>16.2526073455811</v>
+      </c>
+      <c r="O6" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6">
+        <v>-28.9910221099854</v>
+      </c>
+      <c r="Q6">
+        <v>711.9873046875</v>
+      </c>
+      <c r="R6">
+        <v>714.055480957031</v>
+      </c>
+      <c r="S6">
+        <v>713.907104492188</v>
+      </c>
+      <c r="T6">
+        <v>-0.85760498046875</v>
+      </c>
+      <c r="U6">
+        <v>-0.98626708984375</v>
+      </c>
+      <c r="V6">
+        <v>7.7686767578125</v>
+      </c>
+    </row>
+    <row r="7" ht="19.5" customHeight="1">
+      <c r="A7" s="2">
+        <v>46265</v>
+      </c>
+      <c r="B7">
+        <v>1.43621826171875</v>
+      </c>
+      <c r="C7">
+        <v>2.0867919921875</v>
+      </c>
+      <c r="D7">
+        <v>-2.449462890625</v>
+      </c>
+      <c r="E7">
+        <v>715.169982910156</v>
+      </c>
+      <c r="F7">
+        <v>717.580017089844</v>
+      </c>
+      <c r="G7">
+        <v>713.159973144531</v>
+      </c>
+      <c r="H7">
+        <v>716.760009765625</v>
+      </c>
+      <c r="I7">
+        <v>719.753356933594</v>
+      </c>
+      <c r="J7">
+        <v>713.601440429688</v>
+      </c>
+      <c r="K7">
+        <v>32237100</v>
+      </c>
+      <c r="L7">
+        <v>0.409528464078903</v>
+      </c>
+      <c r="M7">
+        <v>64.2447357177734</v>
+      </c>
+      <c r="N7">
+        <v>-10.1967639923096</v>
+      </c>
+      <c r="O7" t="s">
+        <v>23</v>
+      </c>
+      <c r="P7">
+        <v>-4.16709566116333</v>
+      </c>
+      <c r="Q7">
+        <v>716.4013671875</v>
+      </c>
+      <c r="R7">
+        <v>715.804931640625</v>
+      </c>
+      <c r="S7">
+        <v>714.654663085938</v>
+      </c>
+      <c r="T7">
+        <v>2.17333984375</v>
+      </c>
+      <c r="U7">
+        <v>0.44146728515625</v>
+      </c>
+      <c r="V7">
+        <v>6.15191650390625</v>
+      </c>
+    </row>
+    <row r="8" ht="19.5" customHeight="1">
+      <c r="A8" s="2">
+        <v>46262</v>
+      </c>
+      <c r="B8">
+        <v>3.5447998046875</v>
+      </c>
+      <c r="C8">
+        <v>0.5439453125</v>
+      </c>
+      <c r="D8">
+        <v>-3.02606201171875</v>
+      </c>
+      <c r="E8">
+        <v>719.739990234375</v>
+      </c>
+      <c r="F8">
+        <v>724.125</v>
+      </c>
+      <c r="G8">
+        <v>715.085021972656</v>
+      </c>
+      <c r="H8">
+        <v>716.429992675781</v>
+      </c>
+      <c r="I8">
+        <v>719.943054199219</v>
+      </c>
+      <c r="J8">
+        <v>713.0546875</v>
+      </c>
+      <c r="K8">
+        <v>34105300</v>
+      </c>
+      <c r="L8">
+        <v>0.137622654438019</v>
+      </c>
+      <c r="M8">
+        <v>71.5394439697266</v>
+      </c>
+      <c r="N8">
+        <v>-3.5209219455719</v>
+      </c>
+      <c r="O8" t="s">
+        <v>1</v>
+      </c>
+      <c r="P8">
+        <v>0.550081491470337</v>
+      </c>
+      <c r="Q8">
+        <v>716.098693847656</v>
+      </c>
+      <c r="R8">
+        <v>715.528686523438</v>
+      </c>
+      <c r="S8">
+        <v>714.415161132813</v>
+      </c>
+      <c r="T8">
+        <v>-4.18194580078125</v>
+      </c>
+      <c r="U8">
+        <v>-2.03033447265625</v>
+      </c>
+      <c r="V8">
+        <v>6.88836669921875</v>
+      </c>
+    </row>
+    <row r="9" ht="19.5" customHeight="1">
+      <c r="A9" s="2">
+        <v>46261</v>
+      </c>
+      <c r="B9">
+        <v>4.66131591796875</v>
+      </c>
+      <c r="C9">
+        <v>-1.491943359375</v>
+      </c>
+      <c r="D9">
+        <v>-3.8359375</v>
+      </c>
+      <c r="E9">
+        <v>716.929992675781</v>
+      </c>
+      <c r="F9">
+        <v>721.349975585938</v>
+      </c>
+      <c r="G9">
+        <v>714.525024414063</v>
+      </c>
+      <c r="H9">
+        <v>721.109985351563</v>
+      </c>
+      <c r="I9">
+        <v>722.337341308594</v>
+      </c>
+      <c r="J9">
+        <v>717.721252441406</v>
+      </c>
+      <c r="K9">
+        <v>28723400</v>
+      </c>
+      <c r="L9">
+        <v>0.713811993598938</v>
+      </c>
+      <c r="M9">
+        <v>74.1502151489258</v>
+      </c>
+      <c r="N9">
+        <v>-12.5261697769165</v>
+      </c>
+      <c r="O9" t="s">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>35.1892890930176</v>
+      </c>
+      <c r="Q9">
+        <v>715.721313476563</v>
+      </c>
+      <c r="R9">
+        <v>715.231018066406</v>
+      </c>
+      <c r="S9">
+        <v>714.299743652344</v>
+      </c>
+      <c r="T9">
+        <v>0.98736572265625</v>
+      </c>
+      <c r="U9">
+        <v>3.19622802734375</v>
+      </c>
+      <c r="V9">
+        <v>4.6160888671875</v>
+      </c>
+    </row>
+    <row r="10" ht="19.5" customHeight="1">
+      <c r="A10" s="2">
+        <v>46260</v>
+      </c>
+      <c r="B10">
+        <v>0.4306640625</v>
+      </c>
+      <c r="C10">
+        <v>-6.2967529296875</v>
+      </c>
+      <c r="D10">
+        <v>-6.01812744140625</v>
+      </c>
+      <c r="E10">
+        <v>708.409973144531</v>
+      </c>
+      <c r="F10">
+        <v>713.02001953125</v>
+      </c>
+      <c r="G10">
+        <v>707.969970703125</v>
+      </c>
+      <c r="H10">
+        <v>711.369995117188</v>
+      </c>
+      <c r="I10">
+        <v>714.13525390625</v>
+      </c>
+      <c r="J10">
+        <v>708.566284179688</v>
+      </c>
+      <c r="K10">
+        <v>20392300</v>
+      </c>
+      <c r="L10">
+        <v>-0.141427174210548</v>
+      </c>
+      <c r="M10">
+        <v>84.7684555053711</v>
+      </c>
+      <c r="N10">
+        <v>1.23760998249054</v>
+      </c>
+      <c r="O10" t="s">
+        <v>1</v>
+      </c>
+      <c r="P10">
         <v>10.8492841720581</v>
       </c>
-      <c r="Q4">
+      <c r="Q10">
         <v>711.046569824219</v>
       </c>
-      <c r="R4">
+      <c r="R10">
         <v>713.631652832031</v>
       </c>
-      <c r="S4">
+      <c r="S10">
         <v>713.460998535156</v>
       </c>
-      <c r="T4">
+      <c r="T10">
         <v>1.115234375</v>
       </c>
-      <c r="U4">
+      <c r="U10">
         <v>0.5963134765625</v>
       </c>
-      <c r="V4">
+      <c r="V10">
         <v>5.5689697265625</v>
       </c>
     </row>
-    <row r="5" ht="19.5" customHeight="1">
-      <c r="A5" s="1">
+    <row r="11" ht="19.5" customHeight="1">
+      <c r="A11" s="2">
         <v>46259</v>
       </c>
-      <c r="B5">
+      <c r="B11">
         <v>-1.2520751953125</v>
       </c>
-      <c r="C5">
+      <c r="C11">
         <v>-7.48583984375</v>
       </c>
-      <c r="D5">
+      <c r="D11">
         <v>-6.08203125</v>
       </c>
-      <c r="E5">
+      <c r="E11">
         <v>711.219970703125</v>
       </c>
-      <c r="F5">
+      <c r="F11">
         <v>714.039978027344</v>
       </c>
-      <c r="G5">
+      <c r="G11">
         <v>707.450012207031</v>
       </c>
-      <c r="H5">
+      <c r="H11">
         <v>710.719970703125</v>
       </c>
-      <c r="I5">
+      <c r="I11">
         <v>714.233215332031</v>
       </c>
-      <c r="J5">
+      <c r="J11">
         <v>708.015258789063</v>
       </c>
-      <c r="K5">
+      <c r="K11">
         <v>23869600</v>
       </c>
-      <c r="L5">
+      <c r="L11">
         <v>-0.31761822104454</v>
       </c>
-      <c r="M5">
+      <c r="M11">
         <v>83.732177734375</v>
       </c>
-      <c r="N5">
+      <c r="N11">
         <v>9.97407245635986</v>
       </c>
-      <c r="O5" t="s">
+      <c r="O11" t="s">
         <v>1</v>
       </c>
-      <c r="P5">
+      <c r="P11">
         <v>5.51300573348999</v>
       </c>
-      <c r="Q5">
+      <c r="Q11">
         <v>710.73046875</v>
       </c>
-      <c r="R5">
+      <c r="R11">
         <v>714.225708007813</v>
       </c>
-      <c r="S5">
+      <c r="S11">
         <v>713.566101074219</v>
       </c>
-      <c r="T5">
+      <c r="T11">
         <v>0.1932373046875</v>
       </c>
-      <c r="U5">
+      <c r="U11">
         <v>0.56524658203125</v>
       </c>
-      <c r="V5">
+      <c r="V11">
         <v>6.21795654296875</v>
       </c>
     </row>
-    <row r="6" ht="19.5" customHeight="1">
-      <c r="A6" s="1">
+    <row r="12" ht="19.5" customHeight="1">
+      <c r="A12" s="2">
         <v>46258</v>
       </c>
-      <c r="B6">
+      <c r="B12">
         <v>-4.09735107421875</v>
       </c>
-      <c r="C6">
+      <c r="C12">
         <v>-7.77984619140625</v>
       </c>
-      <c r="D6">
+      <c r="D12">
         <v>-6.29669189453125</v>
       </c>
-      <c r="E6">
+      <c r="E12">
         <v>709.659973144531</v>
       </c>
-      <c r="F6">
+      <c r="F12">
         <v>709.789978027344</v>
       </c>
-      <c r="G6">
+      <c r="G12">
         <v>702.700012207031</v>
       </c>
-      <c r="H6">
+      <c r="H12">
         <v>706.320007324219</v>
       </c>
-      <c r="I6">
+      <c r="I12">
         <v>710.232482910156</v>
       </c>
-      <c r="J6">
+      <c r="J12">
         <v>702.45703125</v>
       </c>
-      <c r="K6">
+      <c r="K12">
         <v>37443100</v>
       </c>
-      <c r="L6">
+      <c r="L12">
         <v>-0.749046683311462</v>
       </c>
-      <c r="M6">
+      <c r="M12">
         <v>76.1381072998047</v>
       </c>
-      <c r="N6">
+      <c r="N12">
         <v>-10.0091505050659</v>
       </c>
-      <c r="O6" t="s">
-        <v>21</v>
-      </c>
-      <c r="P6">
+      <c r="O12" t="s">
+        <v>23</v>
+      </c>
+      <c r="P12">
         <v>-22.8135929107666</v>
       </c>
-      <c r="Q6">
+      <c r="Q12">
         <v>710.474365234375</v>
       </c>
-      <c r="R6">
+      <c r="R12">
         <v>715.191345214844</v>
       </c>
-      <c r="S6">
+      <c r="S12">
         <v>713.859497070313</v>
       </c>
-      <c r="T6">
+      <c r="T12">
         <v>0.4425048828125</v>
       </c>
-      <c r="U6">
+      <c r="U12">
         <v>-0.24298095703125</v>
       </c>
-      <c r="V6">
+      <c r="V12">
         <v>7.77545166015625</v>
       </c>
     </row>
-    <row r="7" ht="19.5" customHeight="1">
-      <c r="A7" s="1">
+    <row r="13" ht="19.5" customHeight="1">
+      <c r="A13" s="2">
         <v>46255</v>
       </c>
-      <c r="B7">
+      <c r="B13">
         <v>-3.96600341796875</v>
       </c>
-      <c r="C7">
+      <c r="C13">
         <v>-5.479248046875</v>
       </c>
-      <c r="D7">
+      <c r="D13">
         <v>-2.70074462890625</v>
       </c>
-      <c r="E7">
+      <c r="E13">
         <v>715.22998046875</v>
       </c>
-      <c r="F7">
+      <c r="F13">
         <v>715.673889160156</v>
       </c>
-      <c r="G7">
+      <c r="G13">
         <v>709.200012207031</v>
       </c>
-      <c r="H7">
+      <c r="H13">
         <v>713.440002441406</v>
       </c>
-      <c r="I7">
+      <c r="I13">
         <v>716.713745117188</v>
       </c>
-      <c r="J7">
+      <c r="J13">
         <v>710.5546875</v>
       </c>
-      <c r="K7">
+      <c r="K13">
         <v>33399400</v>
       </c>
-      <c r="L7">
+      <c r="L13">
         <v>-0.884286046028137</v>
       </c>
-      <c r="M7">
+      <c r="M13">
         <v>84.6064987182617</v>
       </c>
-      <c r="N7">
+      <c r="N13">
         <v>48.485767364502</v>
       </c>
-      <c r="O7" t="s">
-        <v>21</v>
-      </c>
-      <c r="P7">
+      <c r="O13" t="s">
+        <v>23</v>
+      </c>
+      <c r="P13">
         <v>-1.74106681346893</v>
       </c>
-      <c r="Q7">
+      <c r="Q13">
         <v>714.61328125</v>
       </c>
-      <c r="R7">
+      <c r="R13">
         <v>717.7197265625</v>
       </c>
-      <c r="S7">
+      <c r="S13">
         <v>714.918212890625</v>
       </c>
-      <c r="T7">
+      <c r="T13">
         <v>1.03985595703125</v>
       </c>
-      <c r="U7">
+      <c r="U13">
         <v>1.35467529296875</v>
       </c>
-      <c r="V7">
+      <c r="V13">
         <v>6.1590576171875</v>
       </c>
     </row>
-    <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="1">
+    <row r="14" ht="19.5" customHeight="1">
+      <c r="A14" s="2">
         <v>46254</v>
       </c>
-      <c r="B8">
+      <c r="B14">
         <v>-7.43365478515625</v>
       </c>
-      <c r="C8">
+      <c r="C14">
         <v>-4.934814453125</v>
       </c>
-      <c r="D8">
+      <c r="D14">
         <v>0.49609375</v>
       </c>
-      <c r="E8">
+      <c r="E14">
         <v>712.090026855469</v>
       </c>
-      <c r="F8">
+      <c r="F14">
         <v>714.940002441406</v>
       </c>
-      <c r="G8">
+      <c r="G14">
         <v>708.52001953125</v>
       </c>
-      <c r="H8">
+      <c r="H14">
         <v>710.929992675781</v>
       </c>
-      <c r="I8">
+      <c r="I14">
         <v>715.544738769531</v>
       </c>
-      <c r="J8">
+      <c r="J14">
         <v>707.915893554688</v>
       </c>
-      <c r="K8">
+      <c r="K14">
         <v>33396400</v>
       </c>
-      <c r="L8">
+      <c r="L14">
         <v>-0.928094744682312</v>
       </c>
-      <c r="M8">
+      <c r="M14">
         <v>56.9795341491699</v>
       </c>
-      <c r="N8">
+      <c r="N14">
         <v>39.8270530700684</v>
       </c>
-      <c r="O8" t="s">
-        <v>21</v>
-      </c>
-      <c r="P8">
+      <c r="O14" t="s">
+        <v>23</v>
+      </c>
+      <c r="P14">
         <v>-14.3682527542114</v>
       </c>
-      <c r="Q8">
+      <c r="Q14">
         <v>715.648803710938</v>
       </c>
-      <c r="R8">
+      <c r="R14">
         <v>718.887145996094</v>
       </c>
-      <c r="S8">
+      <c r="S14">
         <v>715.012329101563</v>
       </c>
-      <c r="T8">
+      <c r="T14">
         <v>0.604736328125</v>
       </c>
-      <c r="U8">
+      <c r="U14">
         <v>-0.6041259765625</v>
       </c>
-      <c r="V8">
+      <c r="V14">
         <v>7.62884521484375</v>
       </c>
     </row>
-    <row r="9" ht="19.5" customHeight="1">
-      <c r="A9" s="1">
+    <row r="15" ht="19.5" customHeight="1">
+      <c r="A15" s="2">
         <v>46253</v>
       </c>
-      <c r="B9">
+      <c r="B15">
         <v>-7.27069091796875</v>
       </c>
-      <c r="C9">
+      <c r="C15">
         <v>-1.59088134765625</v>
       </c>
-      <c r="D9">
+      <c r="D15">
         <v>5.09222412109375</v>
       </c>
-      <c r="E9">
+      <c r="E15">
         <v>720.390014648438</v>
       </c>
-      <c r="F9">
+      <c r="F15">
         <v>721.499816894531</v>
       </c>
-      <c r="G9">
+      <c r="G15">
         <v>712.609985351563</v>
       </c>
-      <c r="H9">
+      <c r="H15">
         <v>716.080017089844</v>
       </c>
-      <c r="I9">
+      <c r="I15">
         <v>720.196044921875</v>
       </c>
-      <c r="J9">
+      <c r="J15">
         <v>712.312255859375</v>
       </c>
-      <c r="K9">
+      <c r="K15">
         <v>35801700</v>
       </c>
-      <c r="L9">
+      <c r="L15">
         <v>-0.790475010871887</v>
       </c>
-      <c r="M9">
+      <c r="M15">
         <v>40.7500076293945</v>
       </c>
-      <c r="N9">
+      <c r="N15">
         <v>-0.867587327957153</v>
       </c>
-      <c r="O9" t="s">
-        <v>21</v>
-      </c>
-      <c r="P9">
+      <c r="O15" t="s">
+        <v>23</v>
+      </c>
+      <c r="P15">
         <v>-27.9632911682129</v>
       </c>
-      <c r="Q9">
+      <c r="Q15">
         <v>719.837768554688</v>
       </c>
-      <c r="R9">
+      <c r="R15">
         <v>720.874938964844</v>
       </c>
-      <c r="S9">
+      <c r="S15">
         <v>715.392578125</v>
       </c>
-      <c r="T9">
+      <c r="T15">
         <v>-1.30377197265625</v>
       </c>
-      <c r="U9">
+      <c r="U15">
         <v>-0.2977294921875</v>
       </c>
-      <c r="V9">
+      <c r="V15">
         <v>7.8837890625</v>
       </c>
     </row>
-    <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="1">
+    <row r="16" ht="19.5" customHeight="1">
+      <c r="A16" s="2">
         <v>46252</v>
       </c>
-      <c r="B10">
+      <c r="B16">
         <v>-5.08782958984375</v>
       </c>
-      <c r="C10">
+      <c r="C16">
         <v>1.26361083984375</v>
       </c>
-      <c r="D10">
+      <c r="D16">
         <v>10.6339111328125</v>
       </c>
-      <c r="E10">
+      <c r="E16">
         <v>720.210021972656</v>
       </c>
-      <c r="F10">
+      <c r="F16">
         <v>722.130004882813</v>
       </c>
-      <c r="G10">
+      <c r="G16">
         <v>715.919982910156</v>
       </c>
-      <c r="H10">
+      <c r="H16">
         <v>717.510009765625</v>
       </c>
-      <c r="I10">
+      <c r="I16">
         <v>721.464477539063</v>
       </c>
-      <c r="J10">
+      <c r="J16">
         <v>713.809631347656</v>
       </c>
-      <c r="K10">
+      <c r="K16">
         <v>48997100</v>
       </c>
-      <c r="L10">
+      <c r="L16">
         <v>-0.470953077077866</v>
       </c>
-      <c r="M10">
+      <c r="M16">
         <v>41.1066436767578</v>
       </c>
-      <c r="N10">
+      <c r="N16">
         <v>41.1687278747559</v>
       </c>
-      <c r="O10" t="s">
-        <v>21</v>
-      </c>
-      <c r="P10">
+      <c r="O16" t="s">
+        <v>23</v>
+      </c>
+      <c r="P16">
         <v>-47.562686920166</v>
       </c>
-      <c r="Q10">
+      <c r="Q16">
         <v>723.48291015625</v>
       </c>
-      <c r="R10">
+      <c r="R16">
         <v>722.074768066406</v>
       </c>
-      <c r="S10">
+      <c r="S16">
         <v>715.1767578125</v>
       </c>
-      <c r="T10">
+      <c r="T16">
         <v>-0.66552734375</v>
       </c>
-      <c r="U10">
+      <c r="U16">
         <v>-2.1103515625</v>
       </c>
-      <c r="V10">
+      <c r="V16">
         <v>7.65484619140625</v>
       </c>
     </row>
-    <row r="11" ht="19.5" customHeight="1">
-      <c r="A11" s="1">
+    <row r="17" ht="19.5" customHeight="1">
+      <c r="A17" s="2">
         <v>46251</v>
       </c>
-      <c r="B11">
+      <c r="B17">
         <v>3.04315185546875</v>
       </c>
-      <c r="C11">
+      <c r="C17">
         <v>4.91015625</v>
       </c>
-      <c r="D11">
+      <c r="D17">
         <v>16.1221923828125</v>
       </c>
-      <c r="E11">
+      <c r="E17">
         <v>732.950012207031</v>
       </c>
-      <c r="F11">
+      <c r="F17">
         <v>734.580017089844</v>
       </c>
-      <c r="G11">
+      <c r="G17">
         <v>729.27001953125</v>
       </c>
-      <c r="H11">
+      <c r="H17">
         <v>729.869995117188</v>
       </c>
-      <c r="I11">
+      <c r="I17">
         <v>733.000610351563</v>
       </c>
-      <c r="J11">
+      <c r="J17">
         <v>727.500427246094</v>
       </c>
-      <c r="K11">
+      <c r="K17">
         <v>26452500</v>
       </c>
-      <c r="L11">
+      <c r="L17">
         <v>-0.632856070995331</v>
       </c>
-      <c r="M11">
+      <c r="M17">
         <v>29.118803024292</v>
       </c>
-      <c r="N11">
+      <c r="N17">
         <v>-30.5778942108154</v>
       </c>
-      <c r="O11" t="s">
-        <v>21</v>
-      </c>
-      <c r="P11">
+      <c r="O17" t="s">
+        <v>23</v>
+      </c>
+      <c r="P17">
         <v>-0.659402906894684</v>
       </c>
-      <c r="Q11">
+      <c r="Q17">
         <v>729.34814453125</v>
       </c>
-      <c r="R11">
+      <c r="R17">
         <v>723.375366210938</v>
       </c>
-      <c r="S11">
+      <c r="S17">
         <v>715.094543457031</v>
       </c>
-      <c r="T11">
+      <c r="T17">
         <v>-1.57940673828125</v>
       </c>
-      <c r="U11">
+      <c r="U17">
         <v>-1.76959228515625</v>
       </c>
-      <c r="V11">
+      <c r="V17">
         <v>5.50018310546875</v>
       </c>
     </row>
-    <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="1">
+    <row r="18" ht="19.5" customHeight="1">
+      <c r="A18" s="2">
         <v>46248</v>
       </c>
-      <c r="B12">
+      <c r="B18">
         <v>4.747802734375</v>
       </c>
-      <c r="C12">
+      <c r="C18">
         <v>7.09246826171875</v>
       </c>
-      <c r="D12">
+      <c r="D18">
         <v>17.9688720703125</v>
       </c>
-      <c r="E12">
+      <c r="E18">
         <v>733.409973144531</v>
       </c>
-      <c r="F12">
+      <c r="F18">
         <v>734.390014648438</v>
       </c>
-      <c r="G12">
+      <c r="G18">
         <v>728.320007324219</v>
       </c>
-      <c r="H12">
+      <c r="H18">
         <v>731.070007324219</v>
       </c>
-      <c r="I12">
+      <c r="I18">
         <v>734.302001953125</v>
       </c>
-      <c r="J12">
+      <c r="J18">
         <v>727.537048339844</v>
       </c>
-      <c r="K12">
+      <c r="K18">
         <v>23790600</v>
       </c>
-      <c r="L12">
+      <c r="L18">
         <v>-0.310950875282288</v>
       </c>
-      <c r="M12">
+      <c r="M18">
         <v>41.9445686340332</v>
       </c>
-      <c r="N12">
+      <c r="N18">
         <v>2.53283834457397</v>
       </c>
-      <c r="O12" t="s">
+      <c r="O18" t="s">
         <v>1</v>
       </c>
-      <c r="P12">
+      <c r="P18">
         <v>12.7733783721924</v>
       </c>
-      <c r="Q12">
+      <c r="Q18">
         <v>728.561706542969</v>
       </c>
-      <c r="R12">
+      <c r="R18">
         <v>721.666564941406</v>
       </c>
-      <c r="S12">
+      <c r="S18">
         <v>713.505493164063</v>
       </c>
-      <c r="T12">
+      <c r="T18">
         <v>-0.0880126953125</v>
       </c>
-      <c r="U12">
+      <c r="U18">
         <v>-0.782958984375</v>
       </c>
-      <c r="V12">
+      <c r="V18">
         <v>6.76495361328125</v>
       </c>
     </row>
-    <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="1">
+    <row r="19" ht="19.5" customHeight="1">
+      <c r="A19" s="2">
         <v>46247</v>
       </c>
-      <c r="B13">
+      <c r="B19">
         <v>4.3778076171875</v>
       </c>
-      <c r="C13">
+      <c r="C19">
         <v>8.908935546875</v>
       </c>
-      <c r="D13">
+      <c r="D19">
         <v>18.5191040039063</v>
       </c>
-      <c r="E13">
+      <c r="E19">
         <v>725.150024414063</v>
       </c>
-      <c r="F13">
+      <c r="F19">
         <v>733.960021972656</v>
       </c>
-      <c r="G13">
+      <c r="G19">
         <v>724.030029296875</v>
       </c>
-      <c r="H13">
+      <c r="H19">
         <v>732.070007324219</v>
       </c>
-      <c r="I13">
+      <c r="I19">
         <v>732.538391113281</v>
       </c>
-      <c r="J13">
+      <c r="J19">
         <v>727.682556152344</v>
       </c>
-      <c r="K13">
+      <c r="K19">
         <v>31599700</v>
       </c>
-      <c r="L13">
+      <c r="L19">
         <v>-0.488571882247925</v>
       </c>
-      <c r="M13">
+      <c r="M19">
         <v>40.9084243774414</v>
       </c>
-      <c r="N13">
+      <c r="N19">
         <v>-31.3219966888428</v>
-      </c>
-      <c r="O13" t="s">
-        <v>1</v>
-      </c>
-      <c r="P13">
-        <v>30.4323463439941</v>
-      </c>
-      <c r="Q13">
-        <v>726.150024414063</v>
-      </c>
-      <c r="R13">
-        <v>718.895812988281</v>
-      </c>
-      <c r="S13">
-        <v>711.396850585938</v>
-      </c>
-      <c r="T13">
-        <v>-1.421630859375</v>
-      </c>
-      <c r="U13">
-        <v>3.65252685546875</v>
-      </c>
-      <c r="V13">
-        <v>4.8558349609375</v>
-      </c>
-    </row>
-    <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="1">
-        <v>46246</v>
-      </c>
-      <c r="B14">
-        <v>2.327392578125</v>
-      </c>
-      <c r="C14">
-        <v>9.25762939453125</v>
-      </c>
-      <c r="D14">
-        <v>17.2620849609375</v>
-      </c>
-      <c r="E14">
-        <v>727.080017089844</v>
-      </c>
-      <c r="F14">
-        <v>727.25</v>
-      </c>
-      <c r="G14">
-        <v>722.919982910156</v>
-      </c>
-      <c r="H14">
-        <v>723.700012207031</v>
-      </c>
-      <c r="I14">
-        <v>726.914245605469</v>
-      </c>
-      <c r="J14">
-        <v>721.6142578125</v>
-      </c>
-      <c r="K14">
-        <v>29065900</v>
-      </c>
-      <c r="L14">
-        <v>-1.10904657840729</v>
-      </c>
-      <c r="M14">
-        <v>59.5655403137207</v>
-      </c>
-      <c r="N14">
-        <v>-8.88726615905762</v>
-      </c>
-      <c r="O14" t="s">
-        <v>1</v>
-      </c>
-      <c r="P14">
-        <v>18.1262340545654</v>
-      </c>
-      <c r="Q14">
-        <v>721.5166015625</v>
-      </c>
-      <c r="R14">
-        <v>715.153076171875</v>
-      </c>
-      <c r="S14">
-        <v>709.211975097656</v>
-      </c>
-      <c r="T14">
-        <v>-0.33575439453125</v>
-      </c>
-      <c r="U14">
-        <v>-1.30572509765625</v>
-      </c>
-      <c r="V14">
-        <v>5.29998779296875</v>
-      </c>
-    </row>
-    <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="1">
-        <v>46245</v>
-      </c>
-      <c r="B15">
-        <v>0.384765625</v>
-      </c>
-      <c r="C15">
-        <v>12.8827514648438</v>
-      </c>
-      <c r="D15">
-        <v>15.763671875</v>
-      </c>
-      <c r="E15">
-        <v>723.289978027344</v>
-      </c>
-      <c r="F15">
-        <v>723.349975585938</v>
-      </c>
-      <c r="G15">
-        <v>715.5</v>
-      </c>
-      <c r="H15">
-        <v>718.450012207031</v>
-      </c>
-      <c r="I15">
-        <v>721.348022460938</v>
-      </c>
-      <c r="J15">
-        <v>715.432067871094</v>
-      </c>
-      <c r="K15">
-        <v>29286100</v>
-      </c>
-      <c r="L15">
-        <v>-0.973330557346344</v>
-      </c>
-      <c r="M15">
-        <v>65.3756484985352</v>
-      </c>
-      <c r="N15">
-        <v>2.9482729434967</v>
-      </c>
-      <c r="O15" t="s">
-        <v>21</v>
-      </c>
-      <c r="P15">
-        <v>-9.89096736907959</v>
-      </c>
-      <c r="Q15">
-        <v>718.969360351563</v>
-      </c>
-      <c r="R15">
-        <v>712.544189453125</v>
-      </c>
-      <c r="S15">
-        <v>707.421081542969</v>
-      </c>
-      <c r="T15">
-        <v>-2.001953125</v>
-      </c>
-      <c r="U15">
-        <v>-0.06793212890625</v>
-      </c>
-      <c r="V15">
-        <v>5.91595458984375</v>
-      </c>
-    </row>
-    <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="1">
-        <v>46244</v>
-      </c>
-      <c r="B16">
-        <v>0.97235107421875</v>
-      </c>
-      <c r="C16">
-        <v>16.9237670898438</v>
-      </c>
-      <c r="D16">
-        <v>15.2864379882813</v>
-      </c>
-      <c r="E16">
-        <v>722.390014648438</v>
-      </c>
-      <c r="F16">
-        <v>724.669982910156</v>
-      </c>
-      <c r="G16">
-        <v>720.330017089844</v>
-      </c>
-      <c r="H16">
-        <v>720.869995117188</v>
-      </c>
-      <c r="I16">
-        <v>724.498474121094</v>
-      </c>
-      <c r="J16">
-        <v>718.993835449219</v>
-      </c>
-      <c r="K16">
-        <v>26243100</v>
-      </c>
-      <c r="L16">
-        <v>-1.02761697769165</v>
-      </c>
-      <c r="M16">
-        <v>63.5033950805664</v>
-      </c>
-      <c r="N16">
-        <v>4.0243992805481</v>
-      </c>
-      <c r="O16" t="s">
-        <v>1</v>
-      </c>
-      <c r="P16">
-        <v>9.99762535095215</v>
-      </c>
-      <c r="Q16">
-        <v>719.53515625</v>
-      </c>
-      <c r="R16">
-        <v>710.855163574219</v>
-      </c>
-      <c r="S16">
-        <v>706.193542480469</v>
-      </c>
-      <c r="T16">
-        <v>-0.1715087890625</v>
-      </c>
-      <c r="U16">
-        <v>-1.336181640625</v>
-      </c>
-      <c r="V16">
-        <v>5.504638671875</v>
-      </c>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="1">
-        <v>46241</v>
-      </c>
-      <c r="B17">
-        <v>4.0394287109375</v>
-      </c>
-      <c r="C17">
-        <v>18.4527587890625</v>
-      </c>
-      <c r="D17">
-        <v>14.3407592773438</v>
-      </c>
-      <c r="E17">
-        <v>720.150024414063</v>
-      </c>
-      <c r="F17">
-        <v>723.630004882813</v>
-      </c>
-      <c r="G17">
-        <v>716.510009765625</v>
-      </c>
-      <c r="H17">
-        <v>723.030029296875</v>
-      </c>
-      <c r="I17">
-        <v>726.10888671875</v>
-      </c>
-      <c r="J17">
-        <v>718.251037597656</v>
-      </c>
-      <c r="K17">
-        <v>31070300</v>
-      </c>
-      <c r="L17">
-        <v>-0.726187586784363</v>
-      </c>
-      <c r="M17">
-        <v>61.0466346740723</v>
-      </c>
-      <c r="N17">
-        <v>-0.528325259685516</v>
-      </c>
-      <c r="O17" t="s">
-        <v>1</v>
-      </c>
-      <c r="P17">
-        <v>26.1653099060059</v>
-      </c>
-      <c r="Q17">
-        <v>717.619018554688</v>
-      </c>
-      <c r="R17">
-        <v>707.809143066406</v>
-      </c>
-      <c r="S17">
-        <v>704.476501464844</v>
-      </c>
-      <c r="T17">
-        <v>2.4788818359375</v>
-      </c>
-      <c r="U17">
-        <v>1.74102783203125</v>
-      </c>
-      <c r="V17">
-        <v>7.85784912109375</v>
-      </c>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="1">
-        <v>46240</v>
-      </c>
-      <c r="B18">
-        <v>5.7655029296875</v>
-      </c>
-      <c r="C18">
-        <v>17.0516967773438</v>
-      </c>
-      <c r="D18">
-        <v>11.1168212890625</v>
-      </c>
-      <c r="E18">
-        <v>710.820007324219</v>
-      </c>
-      <c r="F18">
-        <v>719.320007324219</v>
-      </c>
-      <c r="G18">
-        <v>708.5</v>
-      </c>
-      <c r="H18">
-        <v>714.650024414063</v>
-      </c>
-      <c r="I18">
-        <v>718.173400878906</v>
-      </c>
-      <c r="J18">
-        <v>708.951232910156</v>
-      </c>
-      <c r="K18">
-        <v>33035800</v>
-      </c>
-      <c r="L18">
-        <v>-0.627615809440613</v>
-      </c>
-      <c r="M18">
-        <v>61.3708724975586</v>
-      </c>
-      <c r="N18">
-        <v>-10.5575513839722</v>
-      </c>
-      <c r="O18" t="s">
-        <v>21</v>
-      </c>
-      <c r="P18">
-        <v>-23.3668766021729</v>
-      </c>
-      <c r="Q18">
-        <v>712.781005859375</v>
-      </c>
-      <c r="R18">
-        <v>703.359313964844</v>
-      </c>
-      <c r="S18">
-        <v>702.144226074219</v>
-      </c>
-      <c r="T18">
-        <v>-1.1466064453125</v>
-      </c>
-      <c r="U18">
-        <v>0.45123291015625</v>
-      </c>
-      <c r="V18">
-        <v>9.22216796875</v>
-      </c>
-    </row>
-    <row r="19" ht="19.5" customHeight="1">
-      <c r="A19" s="1">
-        <v>46239</v>
-      </c>
-      <c r="B19">
-        <v>13.2140502929688</v>
-      </c>
-      <c r="C19">
-        <v>17.2907104492188</v>
-      </c>
-      <c r="D19">
-        <v>8.81109619140625</v>
-      </c>
-      <c r="E19">
-        <v>726.25</v>
-      </c>
-      <c r="F19">
-        <v>728.539978027344</v>
-      </c>
-      <c r="G19">
-        <v>716.919982910156</v>
-      </c>
-      <c r="H19">
-        <v>717.299987792969</v>
-      </c>
-      <c r="I19">
-        <v>722.862182617188</v>
-      </c>
-      <c r="J19">
-        <v>712.977844238281</v>
-      </c>
-      <c r="K19">
-        <v>33540100</v>
-      </c>
-      <c r="L19">
-        <v>-0.500950396060944</v>
-      </c>
-      <c r="M19">
-        <v>68.6149291992188</v>
-      </c>
-      <c r="N19">
-        <v>15.4603137969971</v>
       </c>
       <c r="O19" t="s">
         <v>1</v>
       </c>
       <c r="P19">
-        <v>28.8229656219482</v>
+        <v>30.4323463439941</v>
       </c>
       <c r="Q19">
-        <v>711.650634765625</v>
+        <v>726.150024414063</v>
       </c>
       <c r="R19">
-        <v>700.618591308594</v>
+        <v>718.895812988281</v>
       </c>
       <c r="S19">
-        <v>700.785400390625</v>
+        <v>711.396850585938</v>
       </c>
       <c r="T19">
-        <v>-5.67779541015625</v>
+        <v>-1.421630859375</v>
       </c>
       <c r="U19">
-        <v>-3.942138671875</v>
+        <v>3.65252685546875</v>
       </c>
       <c r="V19">
-        <v>9.88433837890625</v>
+        <v>4.8558349609375</v>
       </c>
     </row>
     <row r="20" ht="19.5" customHeight="1">
-      <c r="A20" s="1">
-        <v>46238</v>
+      <c r="A20" s="2">
+        <v>46246</v>
       </c>
       <c r="B20">
-        <v>20.4347534179688</v>
+        <v>2.327392578125</v>
       </c>
       <c r="C20">
-        <v>12.6027221679688</v>
+        <v>9.25762939453125</v>
       </c>
       <c r="D20">
-        <v>3.1591796875</v>
+        <v>17.2620849609375</v>
       </c>
       <c r="E20">
-        <v>708.159973144531</v>
+        <v>727.080017089844</v>
       </c>
       <c r="F20">
-        <v>725.659973144531</v>
+        <v>727.25</v>
       </c>
       <c r="G20">
-        <v>707.530029296875</v>
+        <v>722.919982910156</v>
       </c>
       <c r="H20">
-        <v>723.849975585938</v>
+        <v>723.700012207031</v>
       </c>
       <c r="I20">
-        <v>724.495361328125</v>
+        <v>726.914245605469</v>
       </c>
       <c r="J20">
-        <v>715.428039550781</v>
+        <v>721.6142578125</v>
       </c>
       <c r="K20">
-        <v>59778600</v>
+        <v>29065900</v>
       </c>
       <c r="L20">
-        <v>-0.300473153591156</v>
+        <v>-1.10904657840729</v>
       </c>
       <c r="M20">
-        <v>59.4272842407227</v>
+        <v>59.5655403137207</v>
       </c>
       <c r="N20">
-        <v>-21.2858924865723</v>
+        <v>-8.88726615905762</v>
       </c>
       <c r="O20" t="s">
         <v>1</v>
       </c>
       <c r="P20">
-        <v>100.000007629395</v>
+        <v>18.1262340545654</v>
       </c>
       <c r="Q20">
-        <v>705.591552734375</v>
+        <v>721.5166015625</v>
       </c>
       <c r="R20">
-        <v>695.908142089844</v>
+        <v>715.153076171875</v>
       </c>
       <c r="S20">
-        <v>698.772827148438</v>
+        <v>709.211975097656</v>
       </c>
       <c r="T20">
-        <v>-1.16461181640625</v>
+        <v>-0.33575439453125</v>
       </c>
       <c r="U20">
-        <v>7.89801025390625</v>
+        <v>-1.30572509765625</v>
       </c>
       <c r="V20">
-        <v>9.06732177734375</v>
+        <v>5.29998779296875</v>
       </c>
     </row>
     <row r="21" ht="19.5" customHeight="1">
-      <c r="A21" s="1">
-        <v>46237</v>
+      <c r="A21" s="2">
+        <v>46245</v>
       </c>
       <c r="B21">
-        <v>11.339599609375</v>
+        <v>0.384765625</v>
       </c>
       <c r="C21">
-        <v>0.62603759765625</v>
+        <v>12.8827514648438</v>
       </c>
       <c r="D21">
-        <v>-6.712646484375</v>
+        <v>15.763671875</v>
       </c>
       <c r="E21">
-        <v>688.299987792969</v>
+        <v>723.289978027344</v>
       </c>
       <c r="F21">
-        <v>701.590026855469</v>
+        <v>723.349975585938</v>
       </c>
       <c r="G21">
-        <v>685.820007324219</v>
+        <v>715.5</v>
       </c>
       <c r="H21">
-        <v>700.070007324219</v>
+        <v>718.450012207031</v>
       </c>
       <c r="I21">
-        <v>701.723510742188</v>
+        <v>721.348022460938</v>
       </c>
       <c r="J21">
-        <v>691.503540039063</v>
+        <v>715.432067871094</v>
       </c>
       <c r="K21">
-        <v>44965000</v>
+        <v>29286100</v>
       </c>
       <c r="L21">
-        <v>-0.909996390342712</v>
+        <v>-0.973330557346344</v>
       </c>
       <c r="M21">
-        <v>75.4976272583008</v>
+        <v>65.3756484985352</v>
       </c>
       <c r="N21">
-        <v>-15.1427478790283</v>
+        <v>2.9482729434967</v>
       </c>
       <c r="O21" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P21">
-        <v>66.5761184692383</v>
+        <v>-9.89096736907959</v>
       </c>
       <c r="Q21">
-        <v>689.914428710938</v>
+        <v>718.969360351563</v>
       </c>
       <c r="R21">
-        <v>688.366577148438</v>
+        <v>712.544189453125</v>
       </c>
       <c r="S21">
-        <v>695.902160644531</v>
+        <v>707.421081542969</v>
       </c>
       <c r="T21">
-        <v>0.13348388671875</v>
+        <v>-2.001953125</v>
       </c>
       <c r="U21">
-        <v>5.68353271484375</v>
+        <v>-0.06793212890625</v>
       </c>
       <c r="V21">
-        <v>10.219970703125</v>
+        <v>5.91595458984375</v>
       </c>
     </row>
     <row r="22" ht="19.5" customHeight="1">
-      <c r="A22" s="1">
-        <v>46234</v>
+      <c r="A22" s="2">
+        <v>46244</v>
       </c>
       <c r="B22">
-        <v>5.615966796875</v>
+        <v>0.97235107421875</v>
       </c>
       <c r="C22">
-        <v>-5.2982177734375</v>
+        <v>16.9237670898438</v>
       </c>
       <c r="D22">
-        <v>-11.5888671875</v>
+        <v>15.2864379882813</v>
       </c>
       <c r="E22">
-        <v>692.109985351563</v>
+        <v>722.390014648438</v>
       </c>
       <c r="F22">
-        <v>695.77001953125</v>
+        <v>724.669982910156</v>
       </c>
       <c r="G22">
-        <v>680.051208496094</v>
+        <v>720.330017089844</v>
       </c>
       <c r="H22">
-        <v>687.989990234375</v>
+        <v>720.869995117188</v>
       </c>
       <c r="I22">
-        <v>690.9306640625</v>
+        <v>724.498474121094</v>
       </c>
       <c r="J22">
-        <v>681.263366699219</v>
+        <v>718.993835449219</v>
       </c>
       <c r="K22">
-        <v>50540400</v>
+        <v>26243100</v>
       </c>
       <c r="L22">
-        <v>-2.08857083320618</v>
+        <v>-1.02761697769165</v>
       </c>
       <c r="M22">
-        <v>88.9701538085938</v>
+        <v>63.5033950805664</v>
       </c>
       <c r="N22">
-        <v>2.25866198539734</v>
+        <v>4.0243992805481</v>
       </c>
       <c r="O22" t="s">
         <v>1</v>
       </c>
       <c r="P22">
-        <v>67.7133255004883</v>
+        <v>9.99762535095215</v>
       </c>
       <c r="Q22">
-        <v>682.060668945313</v>
+        <v>719.53515625</v>
       </c>
       <c r="R22">
-        <v>685.576721191406</v>
+        <v>710.855163574219</v>
       </c>
       <c r="S22">
-        <v>695.608276367188</v>
+        <v>706.193542480469</v>
       </c>
       <c r="T22">
-        <v>-4.83935546875</v>
+        <v>-0.1715087890625</v>
       </c>
       <c r="U22">
-        <v>1.212158203125</v>
+        <v>-1.336181640625</v>
       </c>
       <c r="V22">
-        <v>9.66729736328125</v>
+        <v>5.504638671875</v>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1">
-      <c r="A23" s="1">
-        <v>46233</v>
+      <c r="A23" s="2">
+        <v>46241</v>
       </c>
       <c r="B23">
-        <v>0.4974365234375</v>
+        <v>4.0394287109375</v>
       </c>
       <c r="C23">
-        <v>-9.81195068359375</v>
+        <v>18.4527587890625</v>
       </c>
       <c r="D23">
-        <v>-15.7636108398438</v>
+        <v>14.3407592773438</v>
       </c>
       <c r="E23">
-        <v>674.760009765625</v>
+        <v>720.150024414063</v>
       </c>
       <c r="F23">
-        <v>685.119995117188</v>
+        <v>723.630004882813</v>
       </c>
       <c r="G23">
-        <v>673.299987792969</v>
+        <v>716.510009765625</v>
       </c>
       <c r="H23">
-        <v>683.549987792969</v>
+        <v>723.030029296875</v>
       </c>
       <c r="I23">
-        <v>687.009155273438</v>
+        <v>726.10888671875</v>
       </c>
       <c r="J23">
-        <v>678.221374511719</v>
+        <v>718.251037597656</v>
       </c>
       <c r="K23">
-        <v>66753600</v>
+        <v>31070300</v>
       </c>
       <c r="L23">
-        <v>-2.08381009101868</v>
+        <v>-0.726187586784363</v>
       </c>
       <c r="M23">
-        <v>87.0050048828125</v>
+        <v>61.0466346740723</v>
       </c>
       <c r="N23">
-        <v>-12.9949884414673</v>
+        <v>-0.528325259685516</v>
       </c>
       <c r="O23" t="s">
         <v>1</v>
       </c>
       <c r="P23">
-        <v>68.3619155883789</v>
+        <v>26.1653099060059</v>
       </c>
       <c r="Q23">
-        <v>677.404541015625</v>
+        <v>717.619018554688</v>
       </c>
       <c r="R23">
-        <v>684.794189453125</v>
+        <v>707.809143066406</v>
       </c>
       <c r="S23">
-        <v>696.5146484375</v>
+        <v>704.476501464844</v>
       </c>
       <c r="T23">
-        <v>1.88916015625</v>
+        <v>2.4788818359375</v>
       </c>
       <c r="U23">
-        <v>4.92138671875</v>
+        <v>1.74102783203125</v>
       </c>
       <c r="V23">
-        <v>8.78778076171875</v>
+        <v>7.85784912109375</v>
       </c>
     </row>
     <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="1">
-        <v>46232</v>
+      <c r="A24" s="2">
+        <v>46240</v>
       </c>
       <c r="B24">
-        <v>-11.2006225585938</v>
+        <v>5.7655029296875</v>
       </c>
       <c r="C24">
-        <v>-15.3350219726563</v>
+        <v>17.0516967773438</v>
       </c>
       <c r="D24">
-        <v>-19.4429321289063</v>
+        <v>11.1168212890625</v>
       </c>
       <c r="E24">
-        <v>675.510009765625</v>
+        <v>710.820007324219</v>
       </c>
       <c r="F24">
-        <v>680.049987792969</v>
+        <v>719.320007324219</v>
       </c>
       <c r="G24">
-        <v>661.140014648438</v>
+        <v>708.5</v>
       </c>
       <c r="H24">
-        <v>661.72998046875</v>
+        <v>714.650024414063</v>
       </c>
       <c r="I24">
-        <v>670.015625</v>
+        <v>718.173400878906</v>
       </c>
       <c r="J24">
-        <v>656.316345214844</v>
+        <v>708.951232910156</v>
       </c>
       <c r="K24">
-        <v>57233200</v>
+        <v>33035800</v>
       </c>
       <c r="L24">
-        <v>-1.9204740524292</v>
+        <v>-0.627615809440613</v>
       </c>
       <c r="M24">
-        <v>99.9999923706055</v>
+        <v>61.3708724975586</v>
       </c>
       <c r="N24">
-        <v>3.20350408554077</v>
+        <v>-10.5575513839722</v>
       </c>
       <c r="O24" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P24">
-        <v>-68.9146041870117</v>
+        <v>-23.3668766021729</v>
       </c>
       <c r="Q24">
-        <v>671.892639160156</v>
+        <v>712.781005859375</v>
       </c>
       <c r="R24">
-        <v>685.085021972656</v>
+        <v>703.359313964844</v>
       </c>
       <c r="S24">
-        <v>697.902770996094</v>
+        <v>702.144226074219</v>
       </c>
       <c r="T24">
-        <v>-10.0343627929688</v>
+        <v>-1.1466064453125</v>
       </c>
       <c r="U24">
-        <v>-4.82366943359375</v>
+        <v>0.45123291015625</v>
       </c>
       <c r="V24">
-        <v>13.6992797851563</v>
+        <v>9.22216796875</v>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="1">
-        <v>46231</v>
+      <c r="A25" s="2">
+        <v>46239</v>
       </c>
       <c r="B25">
-        <v>-9.48968505859375</v>
+        <v>13.2140502929688</v>
       </c>
       <c r="C25">
-        <v>-12.2387084960938</v>
+        <v>17.2907104492188</v>
       </c>
       <c r="D25">
-        <v>-15.5038452148438</v>
+        <v>8.81109619140625</v>
       </c>
       <c r="E25">
-        <v>676.22998046875</v>
+        <v>726.25</v>
       </c>
       <c r="F25">
-        <v>679.400024414063</v>
+        <v>728.539978027344</v>
       </c>
       <c r="G25">
-        <v>667.880004882813</v>
+        <v>716.919982910156</v>
       </c>
       <c r="H25">
-        <v>675.489990234375</v>
+        <v>717.299987792969</v>
       </c>
       <c r="I25">
-        <v>681.398559570313</v>
+        <v>722.862182617188</v>
       </c>
       <c r="J25">
-        <v>669.311828613281</v>
+        <v>712.977844238281</v>
       </c>
       <c r="K25">
-        <v>51398700</v>
+        <v>33540100</v>
       </c>
       <c r="L25">
-        <v>-0.783804774284363</v>
+        <v>-0.500950396060944</v>
       </c>
       <c r="M25">
-        <v>96.8959274291992</v>
+        <v>68.6149291992188</v>
       </c>
       <c r="N25">
-        <v>5.64116907119751</v>
+        <v>15.4603137969971</v>
       </c>
       <c r="O25" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P25">
-        <v>-45.0695037841797</v>
+        <v>28.8229656219482</v>
       </c>
       <c r="Q25">
-        <v>681.100524902344</v>
+        <v>711.650634765625</v>
       </c>
       <c r="R25">
-        <v>691.612365722656</v>
+        <v>700.618591308594</v>
       </c>
       <c r="S25">
-        <v>701.984680175781</v>
+        <v>700.785400390625</v>
       </c>
       <c r="T25">
-        <v>1.99853515625</v>
+        <v>-5.67779541015625</v>
       </c>
       <c r="U25">
-        <v>1.43182373046875</v>
+        <v>-3.942138671875</v>
       </c>
       <c r="V25">
-        <v>12.0867309570313</v>
+        <v>9.88433837890625</v>
       </c>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="1">
-        <v>46230</v>
+      <c r="A26" s="2">
+        <v>46238</v>
       </c>
       <c r="B26">
-        <v>-10.3001098632813</v>
+        <v>20.4347534179688</v>
       </c>
       <c r="C26">
-        <v>-11.3073120117188</v>
+        <v>12.6027221679688</v>
       </c>
       <c r="D26">
-        <v>-12.7749633789063</v>
+        <v>3.1591796875</v>
       </c>
       <c r="E26">
-        <v>691.679992675781</v>
+        <v>708.159973144531</v>
       </c>
       <c r="F26">
-        <v>692.299987792969</v>
+        <v>725.659973144531</v>
       </c>
       <c r="G26">
-        <v>675.945007324219</v>
+        <v>707.530029296875</v>
       </c>
       <c r="H26">
-        <v>682.119995117188</v>
+        <v>723.849975585938</v>
       </c>
       <c r="I26">
-        <v>687.197937011719</v>
+        <v>724.495361328125</v>
       </c>
       <c r="J26">
-        <v>676.772521972656</v>
+        <v>715.428039550781</v>
       </c>
       <c r="K26">
-        <v>42681400</v>
+        <v>59778600</v>
       </c>
       <c r="L26">
-        <v>-0.777614057064056</v>
+        <v>-0.300473153591156</v>
       </c>
       <c r="M26">
-        <v>91.7217483520508</v>
+        <v>59.4272842407227</v>
       </c>
       <c r="N26">
-        <v>28.3568496704102</v>
+        <v>-21.2858924865723</v>
       </c>
       <c r="O26" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P26">
-        <v>-35.6940422058105</v>
+        <v>100.000007629395</v>
       </c>
       <c r="Q26">
-        <v>686.793579101563</v>
+        <v>705.591552734375</v>
       </c>
       <c r="R26">
-        <v>696.032958984375</v>
+        <v>695.908142089844</v>
       </c>
       <c r="S26">
-        <v>705.08837890625</v>
+        <v>698.772827148438</v>
       </c>
       <c r="T26">
-        <v>-5.10205078125</v>
+        <v>-1.16461181640625</v>
       </c>
       <c r="U26">
-        <v>0.8275146484375</v>
+        <v>7.89801025390625</v>
       </c>
       <c r="V26">
-        <v>10.4254150390625</v>
+        <v>9.06732177734375</v>
       </c>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="1">
-        <v>46227</v>
+      <c r="A27" s="2">
+        <v>46237</v>
       </c>
       <c r="B27">
-        <v>-8.69158935546875</v>
+        <v>11.339599609375</v>
       </c>
       <c r="C27">
-        <v>-9.875</v>
+        <v>0.62603759765625</v>
       </c>
       <c r="D27">
-        <v>-11.1927490234375</v>
+        <v>-6.712646484375</v>
       </c>
       <c r="E27">
-        <v>690.409973144531</v>
+        <v>688.299987792969</v>
       </c>
       <c r="F27">
-        <v>692.630004882813</v>
+        <v>701.590026855469</v>
       </c>
       <c r="G27">
-        <v>682.47998046875</v>
+        <v>685.820007324219</v>
       </c>
       <c r="H27">
-        <v>684.22998046875</v>
+        <v>700.070007324219</v>
       </c>
       <c r="I27">
-        <v>690.563537597656</v>
+        <v>701.723510742188</v>
       </c>
       <c r="J27">
-        <v>679.935974121094</v>
+        <v>691.503540039063</v>
       </c>
       <c r="K27">
-        <v>42876600</v>
+        <v>44965000</v>
       </c>
       <c r="L27">
-        <v>-0.775710344314575</v>
+        <v>-0.909996390342712</v>
       </c>
       <c r="M27">
-        <v>71.4583969116211</v>
+        <v>75.4976272583008</v>
       </c>
       <c r="N27">
-        <v>26.3548107147217</v>
+        <v>-15.1427478790283</v>
       </c>
       <c r="O27" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P27">
-        <v>-63.8044128417969</v>
+        <v>66.5761184692383</v>
       </c>
       <c r="Q27">
-        <v>691.569458007813</v>
+        <v>689.914428710938</v>
       </c>
       <c r="R27">
-        <v>699.823181152344</v>
+        <v>688.366577148438</v>
       </c>
       <c r="S27">
-        <v>707.758605957031</v>
+        <v>695.902160644531</v>
       </c>
       <c r="T27">
-        <v>-2.06646728515625</v>
+        <v>0.13348388671875</v>
       </c>
       <c r="U27">
-        <v>-2.54400634765625</v>
+        <v>5.68353271484375</v>
       </c>
       <c r="V27">
-        <v>10.6275634765625</v>
+        <v>10.219970703125</v>
       </c>
     </row>
     <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="1">
-        <v>46226</v>
+      <c r="A28" s="2">
+        <v>46234</v>
       </c>
       <c r="B28">
-        <v>-3.48541259765625</v>
+        <v>5.615966796875</v>
       </c>
       <c r="C28">
-        <v>-8.06353759765625</v>
+        <v>-5.2982177734375</v>
       </c>
       <c r="D28">
-        <v>-8.079833984375</v>
+        <v>-11.5888671875</v>
       </c>
       <c r="E28">
-        <v>694.669982910156</v>
+        <v>692.109985351563</v>
       </c>
       <c r="F28">
-        <v>698.659973144531</v>
+        <v>695.77001953125</v>
       </c>
       <c r="G28">
-        <v>687.789978027344</v>
+        <v>680.051208496094</v>
       </c>
       <c r="H28">
-        <v>691.960021972656</v>
+        <v>687.989990234375</v>
       </c>
       <c r="I28">
-        <v>696.182250976563</v>
+        <v>690.9306640625</v>
       </c>
       <c r="J28">
-        <v>686.057800292969</v>
+        <v>681.263366699219</v>
       </c>
       <c r="K28">
-        <v>44028500</v>
+        <v>50540400</v>
       </c>
       <c r="L28">
-        <v>-0.707615435123444</v>
+        <v>-2.08857083320618</v>
       </c>
       <c r="M28">
-        <v>56.5537605285645</v>
+        <v>88.9701538085938</v>
       </c>
       <c r="N28">
-        <v>7.45290517807007</v>
+        <v>2.25866198539734</v>
       </c>
       <c r="O28" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P28">
-        <v>-56.6292991638184</v>
+        <v>67.7133255004883</v>
       </c>
       <c r="Q28">
-        <v>698.227111816406</v>
+        <v>682.060668945313</v>
       </c>
       <c r="R28">
-        <v>704.183776855469</v>
+        <v>685.576721191406</v>
       </c>
       <c r="S28">
-        <v>710.521728515625</v>
+        <v>695.608276367188</v>
       </c>
       <c r="T28">
-        <v>-2.47772216796875</v>
+        <v>-4.83935546875</v>
       </c>
       <c r="U28">
-        <v>-1.732177734375</v>
+        <v>1.212158203125</v>
       </c>
       <c r="V28">
-        <v>10.1244506835938</v>
+        <v>9.66729736328125</v>
       </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="1">
-        <v>46225</v>
+      <c r="A29" s="2">
+        <v>46233</v>
       </c>
       <c r="B29">
-        <v>3.01220703125</v>
+        <v>0.4974365234375</v>
       </c>
       <c r="C29">
-        <v>-5.4625244140625</v>
+        <v>-9.81195068359375</v>
       </c>
       <c r="D29">
-        <v>-6.10992431640625</v>
+        <v>-15.7636108398438</v>
       </c>
       <c r="E29">
-        <v>703.619995117188</v>
+        <v>674.760009765625</v>
       </c>
       <c r="F29">
-        <v>709.650024414063</v>
+        <v>685.119995117188</v>
       </c>
       <c r="G29">
-        <v>703.619995117188</v>
+        <v>673.299987792969</v>
       </c>
       <c r="H29">
-        <v>705.349975585938</v>
+        <v>683.549987792969</v>
       </c>
       <c r="I29">
-        <v>708.769348144531</v>
+        <v>687.009155273438</v>
       </c>
       <c r="J29">
-        <v>701.754638671875</v>
+        <v>678.221374511719</v>
       </c>
       <c r="K29">
-        <v>23692100</v>
+        <v>66753600</v>
       </c>
       <c r="L29">
-        <v>-0.678091883659363</v>
+        <v>-2.08381009101868</v>
       </c>
       <c r="M29">
-        <v>52.6312065124512</v>
+        <v>87.0050048828125</v>
       </c>
       <c r="N29">
-        <v>-15.308910369873</v>
+        <v>-12.9949884414673</v>
       </c>
       <c r="O29" t="s">
         <v>1</v>
       </c>
       <c r="P29">
-        <v>10.9916353225708</v>
+        <v>68.3619155883789</v>
       </c>
       <c r="Q29">
-        <v>705.042114257813</v>
+        <v>677.404541015625</v>
       </c>
       <c r="R29">
-        <v>707.900085449219</v>
+        <v>684.794189453125</v>
       </c>
       <c r="S29">
-        <v>712.692932128906</v>
+        <v>696.5146484375</v>
       </c>
       <c r="T29">
-        <v>-0.88067626953125</v>
+        <v>1.88916015625</v>
       </c>
       <c r="U29">
-        <v>-1.8653564453125</v>
+        <v>4.92138671875</v>
       </c>
       <c r="V29">
-        <v>7.01470947265625</v>
+        <v>8.78778076171875</v>
       </c>
     </row>
     <row r="30" ht="19.5" customHeight="1">
-      <c r="A30" s="1">
-        <v>46224</v>
+      <c r="A30" s="2">
+        <v>46232</v>
       </c>
       <c r="B30">
-        <v>0.6416015625</v>
+        <v>-11.2006225585938</v>
       </c>
       <c r="C30">
-        <v>-6.202392578125</v>
+        <v>-15.3350219726563</v>
       </c>
       <c r="D30">
-        <v>-7.814697265625</v>
+        <v>-19.4429321289063</v>
       </c>
       <c r="E30">
-        <v>706.570007324219</v>
+        <v>675.510009765625</v>
       </c>
       <c r="F30">
-        <v>710.049987792969</v>
+        <v>680.049987792969</v>
       </c>
       <c r="G30">
-        <v>702.799987792969</v>
+        <v>661.140014648438</v>
       </c>
       <c r="H30">
-        <v>708.969970703125</v>
+        <v>661.72998046875</v>
       </c>
       <c r="I30">
-        <v>712.483276367188</v>
+        <v>670.015625</v>
       </c>
       <c r="J30">
-        <v>705.233276367188</v>
+        <v>656.316345214844</v>
       </c>
       <c r="K30">
-        <v>33728300</v>
+        <v>57233200</v>
       </c>
       <c r="L30">
-        <v>-0.954281747341156</v>
+        <v>-1.9204740524292</v>
       </c>
       <c r="M30">
-        <v>62.1449165344238</v>
+        <v>99.9999923706055</v>
       </c>
       <c r="N30">
-        <v>-6.62933874130249</v>
+        <v>3.20350408554077</v>
       </c>
       <c r="O30" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P30">
-        <v>48.3449096679688</v>
+        <v>-68.9146041870117</v>
       </c>
       <c r="Q30">
-        <v>704.79150390625</v>
+        <v>671.892639160156</v>
       </c>
       <c r="R30">
-        <v>708.46826171875</v>
+        <v>685.085021972656</v>
       </c>
       <c r="S30">
-        <v>713.447265625</v>
+        <v>697.902770996094</v>
       </c>
       <c r="T30">
-        <v>2.43328857421875</v>
+        <v>-10.0343627929688</v>
       </c>
       <c r="U30">
-        <v>2.43328857421875</v>
+        <v>-4.82366943359375</v>
       </c>
       <c r="V30">
-        <v>7.25</v>
+        <v>13.6992797851563</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1">
-      <c r="A31" s="1">
-        <v>46223</v>
+      <c r="A31" s="2">
+        <v>46231</v>
       </c>
       <c r="B31">
-        <v>-8.39520263671875</v>
+        <v>-9.48968505859375</v>
       </c>
       <c r="C31">
-        <v>-8.765380859375</v>
+        <v>-12.2387084960938</v>
       </c>
       <c r="D31">
-        <v>-9.8062744140625</v>
+        <v>-15.5038452148438</v>
       </c>
       <c r="E31">
-        <v>702.159973144531</v>
+        <v>676.22998046875</v>
       </c>
       <c r="F31">
-        <v>705.799987792969</v>
+        <v>679.400024414063</v>
       </c>
       <c r="G31">
-        <v>695.510009765625</v>
+        <v>667.880004882813</v>
       </c>
       <c r="H31">
-        <v>696.059997558594</v>
+        <v>675.489990234375</v>
       </c>
       <c r="I31">
-        <v>703.789184570313</v>
+        <v>681.398559570313</v>
       </c>
       <c r="J31">
-        <v>693.406494140625</v>
+        <v>669.311828613281</v>
       </c>
       <c r="K31">
-        <v>29687500</v>
+        <v>51398700</v>
       </c>
       <c r="L31">
-        <v>-0.905709385871887</v>
+        <v>-0.783804774284363</v>
       </c>
       <c r="M31">
-        <v>66.5572204589844</v>
+        <v>96.8959274291992</v>
       </c>
       <c r="N31">
-        <v>22.5973968505859</v>
+        <v>5.64116907119751</v>
       </c>
       <c r="O31" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P31">
-        <v>-6.00122213363647</v>
+        <v>-45.0695037841797</v>
       </c>
       <c r="Q31">
-        <v>700.701416015625</v>
+        <v>681.100524902344</v>
       </c>
       <c r="R31">
-        <v>708.291809082031</v>
+        <v>691.612365722656</v>
       </c>
       <c r="S31">
-        <v>713.96923828125</v>
+        <v>701.984680175781</v>
       </c>
       <c r="T31">
-        <v>-2.01080322265625</v>
+        <v>1.99853515625</v>
       </c>
       <c r="U31">
-        <v>-2.103515625</v>
+        <v>1.43182373046875</v>
       </c>
       <c r="V31">
-        <v>10.3826904296875</v>
+        <v>12.0867309570313</v>
       </c>
     </row>
     <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" s="1">
-        <v>46220</v>
+      <c r="A32" s="2">
+        <v>46230</v>
       </c>
       <c r="B32">
-        <v>-9.927001953125</v>
+        <v>-10.3001098632813</v>
       </c>
       <c r="C32">
-        <v>-7.9847412109375</v>
+        <v>-11.3073120117188</v>
       </c>
       <c r="D32">
-        <v>-7.42694091796875</v>
+        <v>-12.7749633789063</v>
       </c>
       <c r="E32">
-        <v>691.650024414063</v>
+        <v>691.679992675781</v>
       </c>
       <c r="F32">
-        <v>702.299987792969</v>
+        <v>692.299987792969</v>
       </c>
       <c r="G32">
-        <v>686.760009765625</v>
+        <v>675.945007324219</v>
       </c>
       <c r="H32">
-        <v>695.330017089844</v>
+        <v>682.119995117188</v>
       </c>
       <c r="I32">
-        <v>701.341003417969</v>
+        <v>687.197937011719</v>
       </c>
       <c r="J32">
-        <v>688.661193847656</v>
+        <v>676.772521972656</v>
       </c>
       <c r="K32">
-        <v>54109200</v>
+        <v>42681400</v>
       </c>
       <c r="L32">
-        <v>-1.21904349327087</v>
+        <v>-0.777614057064056</v>
       </c>
       <c r="M32">
-        <v>54.2892608642578</v>
+        <v>91.7217483520508</v>
       </c>
       <c r="N32">
-        <v>8.37738990783691</v>
+        <v>28.3568496704102</v>
       </c>
       <c r="O32" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P32">
-        <v>-64.7480239868164</v>
+        <v>-35.6940422058105</v>
       </c>
       <c r="Q32">
-        <v>703.639892578125</v>
+        <v>686.793579101563</v>
       </c>
       <c r="R32">
-        <v>711.3662109375</v>
+        <v>696.032958984375</v>
       </c>
       <c r="S32">
-        <v>715.791137695313</v>
+        <v>705.08837890625</v>
       </c>
       <c r="T32">
-        <v>-0.958984375</v>
+        <v>-5.10205078125</v>
       </c>
       <c r="U32">
-        <v>1.90118408203125</v>
+        <v>0.8275146484375</v>
       </c>
       <c r="V32">
-        <v>12.6798095703125</v>
+        <v>10.4254150390625</v>
       </c>
     </row>
     <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="1">
-        <v>46219</v>
+      <c r="A33" s="2">
+        <v>46227</v>
       </c>
       <c r="B33">
-        <v>-5.863037109375</v>
+        <v>-8.69158935546875</v>
       </c>
       <c r="C33">
-        <v>-2.36517333984375</v>
+        <v>-9.875</v>
       </c>
       <c r="D33">
-        <v>-3.09661865234375</v>
+        <v>-11.1927490234375</v>
       </c>
       <c r="E33">
-        <v>712.010009765625</v>
+        <v>690.409973144531</v>
       </c>
       <c r="F33">
-        <v>713.598999023438</v>
+        <v>692.630004882813</v>
       </c>
       <c r="G33">
-        <v>702.609985351563</v>
+        <v>682.47998046875</v>
       </c>
       <c r="H33">
-        <v>705.940002441406</v>
+        <v>684.22998046875</v>
       </c>
       <c r="I33">
-        <v>712.521850585938</v>
+        <v>690.563537597656</v>
       </c>
       <c r="J33">
-        <v>701.248962402344</v>
+        <v>679.935974121094</v>
       </c>
       <c r="K33">
-        <v>39402000</v>
+        <v>42876600</v>
       </c>
       <c r="L33">
-        <v>-1.98428201675415</v>
+        <v>-0.775710344314575</v>
       </c>
       <c r="M33">
-        <v>50.0927925109863</v>
+        <v>71.4583969116211</v>
       </c>
       <c r="N33">
-        <v>7.75767660140991</v>
+        <v>26.3548107147217</v>
       </c>
       <c r="O33" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P33">
-        <v>-43.6580963134766</v>
+        <v>-63.8044128417969</v>
       </c>
       <c r="Q33">
-        <v>712.182556152344</v>
+        <v>691.569458007813</v>
       </c>
       <c r="R33">
-        <v>715.892822265625</v>
+        <v>699.823181152344</v>
       </c>
       <c r="S33">
-        <v>718.15576171875</v>
+        <v>707.758605957031</v>
       </c>
       <c r="T33">
-        <v>-1.0771484375</v>
+        <v>-2.06646728515625</v>
       </c>
       <c r="U33">
-        <v>-1.36102294921875</v>
+        <v>-2.54400634765625</v>
       </c>
       <c r="V33">
-        <v>11.2728881835938</v>
+        <v>10.6275634765625</v>
       </c>
     </row>
     <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="1">
-        <v>46218</v>
+      <c r="A34" s="2">
+        <v>46226</v>
       </c>
       <c r="B34">
-        <v>-1.943359375</v>
+        <v>-3.48541259765625</v>
       </c>
       <c r="C34">
-        <v>0.40814208984375</v>
+        <v>-8.06353759765625</v>
       </c>
       <c r="D34">
-        <v>-0.0054931640625</v>
+        <v>-8.079833984375</v>
       </c>
       <c r="E34">
-        <v>723.849975585938</v>
+        <v>694.669982910156</v>
       </c>
       <c r="F34">
-        <v>724.359985351563</v>
+        <v>698.659973144531</v>
       </c>
       <c r="G34">
-        <v>710.22998046875</v>
+        <v>687.789978027344</v>
       </c>
       <c r="H34">
-        <v>717.739990234375</v>
+        <v>691.960021972656</v>
       </c>
       <c r="I34">
-        <v>721.251037597656</v>
+        <v>696.182250976563</v>
       </c>
       <c r="J34">
-        <v>712.604736328125</v>
+        <v>686.057800292969</v>
       </c>
       <c r="K34">
-        <v>32627500</v>
+        <v>44028500</v>
       </c>
       <c r="L34">
-        <v>-1.41428053379059</v>
+        <v>-0.707615435123444</v>
       </c>
       <c r="M34">
-        <v>46.4865188598633</v>
+        <v>56.5537605285645</v>
       </c>
       <c r="N34">
-        <v>-4.76508235931396</v>
+        <v>7.45290517807007</v>
       </c>
       <c r="O34" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P34">
-        <v>-2.18429470062256</v>
+        <v>-56.6292991638184</v>
       </c>
       <c r="Q34">
-        <v>717.8037109375</v>
+        <v>698.227111816406</v>
       </c>
       <c r="R34">
-        <v>718.531005859375</v>
+        <v>704.183776855469</v>
       </c>
       <c r="S34">
-        <v>719.552307128906</v>
+        <v>710.521728515625</v>
       </c>
       <c r="T34">
-        <v>-3.10894775390625</v>
+        <v>-2.47772216796875</v>
       </c>
       <c r="U34">
-        <v>2.374755859375</v>
+        <v>-1.732177734375</v>
       </c>
       <c r="V34">
-        <v>8.64630126953125</v>
+        <v>10.1244506835938</v>
       </c>
     </row>
     <row r="35" ht="19.5" customHeight="1">
-      <c r="A35" s="1">
-        <v>46217</v>
+      <c r="A35" s="2">
+        <v>46225</v>
       </c>
       <c r="B35">
-        <v>0.21160888671875</v>
+        <v>3.01220703125</v>
       </c>
       <c r="C35">
-        <v>-1.59527587890625</v>
+        <v>-5.4625244140625</v>
       </c>
       <c r="D35">
-        <v>0.46612548828125</v>
+        <v>-6.10992431640625</v>
       </c>
       <c r="E35">
-        <v>720.219970703125</v>
+        <v>703.619995117188</v>
       </c>
       <c r="F35">
-        <v>722.289978027344</v>
+        <v>709.650024414063</v>
       </c>
       <c r="G35">
-        <v>714.340026855469</v>
+        <v>703.619995117188</v>
       </c>
       <c r="H35">
-        <v>719.690002441406</v>
+        <v>705.349975585938</v>
       </c>
       <c r="I35">
-        <v>723.544555664063</v>
+        <v>708.769348144531</v>
       </c>
       <c r="J35">
-        <v>716.334533691406</v>
+        <v>701.754638671875</v>
       </c>
       <c r="K35">
-        <v>29448100</v>
+        <v>23692100</v>
       </c>
       <c r="L35">
-        <v>-0.94570779800415</v>
+        <v>-0.678091883659363</v>
       </c>
       <c r="M35">
-        <v>48.8124732971191</v>
+        <v>52.6312065124512</v>
       </c>
       <c r="N35">
-        <v>-5.16571569442749</v>
+        <v>-15.308910369873</v>
       </c>
       <c r="O35" t="s">
         <v>1</v>
       </c>
       <c r="P35">
-        <v>5.93372297286987</v>
+        <v>10.9916353225708</v>
       </c>
       <c r="Q35">
-        <v>718.3955078125</v>
+        <v>705.042114257813</v>
       </c>
       <c r="R35">
-        <v>718.438903808594</v>
+        <v>707.900085449219</v>
       </c>
       <c r="S35">
-        <v>719.708923339844</v>
+        <v>712.692932128906</v>
       </c>
       <c r="T35">
-        <v>1.25457763671875</v>
+        <v>-0.88067626953125</v>
       </c>
       <c r="U35">
-        <v>1.9945068359375</v>
+        <v>-1.8653564453125</v>
       </c>
       <c r="V35">
-        <v>7.21002197265625</v>
+        <v>7.01470947265625</v>
       </c>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="1">
-        <v>46216</v>
+      <c r="A36" s="2">
+        <v>46224</v>
       </c>
       <c r="B36">
-        <v>-0.3555908203125</v>
+        <v>0.6416015625</v>
       </c>
       <c r="C36">
-        <v>-3.0672607421875</v>
+        <v>-6.202392578125</v>
       </c>
       <c r="D36">
-        <v>-1.38330078125</v>
+        <v>-7.814697265625</v>
       </c>
       <c r="E36">
-        <v>717.719970703125</v>
+        <v>706.570007324219</v>
       </c>
       <c r="F36">
-        <v>718.739990234375</v>
+        <v>710.049987792969</v>
       </c>
       <c r="G36">
-        <v>710.080017089844</v>
+        <v>702.799987792969</v>
       </c>
       <c r="H36">
-        <v>711.739990234375</v>
+        <v>708.969970703125</v>
       </c>
       <c r="I36">
-        <v>717.577209472656</v>
+        <v>712.483276367188</v>
       </c>
       <c r="J36">
-        <v>707.793212890625</v>
+        <v>705.233276367188</v>
       </c>
       <c r="K36">
-        <v>36552300</v>
+        <v>33728300</v>
       </c>
       <c r="L36">
-        <v>-0.0714227557182312</v>
+        <v>-0.954281747341156</v>
       </c>
       <c r="M36">
-        <v>51.4713363647461</v>
+        <v>62.1449165344238</v>
       </c>
       <c r="N36">
-        <v>4.72496747970581</v>
+        <v>-6.62933874130249</v>
       </c>
       <c r="O36" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P36">
-        <v>-42.1362648010254</v>
+        <v>48.3449096679688</v>
       </c>
       <c r="Q36">
-        <v>716.920593261719</v>
+        <v>704.79150390625</v>
       </c>
       <c r="R36">
-        <v>718.116577148438</v>
+        <v>708.46826171875</v>
       </c>
       <c r="S36">
-        <v>719.618469238281</v>
+        <v>713.447265625</v>
       </c>
       <c r="T36">
-        <v>-1.16278076171875</v>
+        <v>2.43328857421875</v>
       </c>
       <c r="U36">
-        <v>-2.28680419921875</v>
+        <v>2.43328857421875</v>
       </c>
       <c r="V36">
-        <v>9.78399658203125</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="37" ht="19.5" customHeight="1">
-      <c r="A37" s="1">
-        <v>46213</v>
+      <c r="A37" s="2">
+        <v>46223</v>
       </c>
       <c r="B37">
-        <v>4.54119873046875</v>
+        <v>-8.39520263671875</v>
       </c>
       <c r="C37">
-        <v>1.09893798828125</v>
+        <v>-8.765380859375</v>
       </c>
       <c r="D37">
-        <v>-0.62530517578125</v>
+        <v>-9.8062744140625</v>
       </c>
       <c r="E37">
-        <v>720.700012207031</v>
+        <v>702.159973144531</v>
       </c>
       <c r="F37">
-        <v>726.390014648438</v>
+        <v>705.799987792969</v>
       </c>
       <c r="G37">
-        <v>717</v>
+        <v>695.510009765625</v>
       </c>
       <c r="H37">
-        <v>725.510009765625</v>
+        <v>696.059997558594</v>
       </c>
       <c r="I37">
-        <v>728.048034667969</v>
+        <v>703.789184570313</v>
       </c>
       <c r="J37">
-        <v>721.283996582031</v>
+        <v>693.406494140625</v>
       </c>
       <c r="K37">
-        <v>26415900</v>
+        <v>29687500</v>
       </c>
       <c r="L37">
-        <v>-0.166184201836586</v>
+        <v>-0.905709385871887</v>
       </c>
       <c r="M37">
-        <v>49.1490592956543</v>
+        <v>66.5572204589844</v>
       </c>
       <c r="N37">
-        <v>-9.55446624755859</v>
+        <v>22.5973968505859</v>
       </c>
       <c r="O37" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P37">
-        <v>29.1831836700439</v>
+        <v>-6.00122213363647</v>
       </c>
       <c r="Q37">
-        <v>721.479248046875</v>
+        <v>700.701416015625</v>
       </c>
       <c r="R37">
-        <v>719.98193359375</v>
+        <v>708.291809082031</v>
       </c>
       <c r="S37">
-        <v>720.620422363281</v>
+        <v>713.96923828125</v>
       </c>
       <c r="T37">
-        <v>1.65802001953125</v>
+        <v>-2.01080322265625</v>
       </c>
       <c r="U37">
-        <v>4.28399658203125</v>
+        <v>-2.103515625</v>
       </c>
       <c r="V37">
-        <v>6.7640380859375</v>
+        <v>10.3826904296875</v>
       </c>
     </row>
     <row r="38" ht="19.5" customHeight="1">
-      <c r="A38" s="1">
-        <v>46212</v>
+      <c r="A38" s="2">
+        <v>46220</v>
       </c>
       <c r="B38">
-        <v>3.296630859375</v>
+        <v>-9.927001953125</v>
       </c>
       <c r="C38">
-        <v>-0.72021484375</v>
+        <v>-7.9847412109375</v>
       </c>
       <c r="D38">
-        <v>-2.30474853515625</v>
+        <v>-7.42694091796875</v>
       </c>
       <c r="E38">
-        <v>718.330017089844</v>
+        <v>691.650024414063</v>
       </c>
       <c r="F38">
-        <v>724.22998046875</v>
+        <v>702.299987792969</v>
       </c>
       <c r="G38">
-        <v>715.125</v>
+        <v>686.760009765625</v>
       </c>
       <c r="H38">
-        <v>723.280029296875</v>
+        <v>695.330017089844</v>
       </c>
       <c r="I38">
-        <v>726.686767578125</v>
+        <v>701.341003417969</v>
       </c>
       <c r="J38">
-        <v>719.118225097656</v>
+        <v>688.661193847656</v>
       </c>
       <c r="K38">
-        <v>33654700</v>
+        <v>54109200</v>
       </c>
       <c r="L38">
-        <v>-1.11665856838226</v>
+        <v>-1.21904349327087</v>
       </c>
       <c r="M38">
-        <v>54.3410568237305</v>
+        <v>54.2892608642578</v>
       </c>
       <c r="N38">
-        <v>-1.37647461891174</v>
+        <v>8.37738990783691</v>
       </c>
       <c r="O38" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="P38">
-        <v>56.2780990600586</v>
+        <v>-64.7480239868164</v>
       </c>
       <c r="Q38">
-        <v>718.006164550781</v>
+        <v>703.639892578125</v>
       </c>
       <c r="R38">
-        <v>718.503051757813</v>
+        <v>711.3662109375</v>
       </c>
       <c r="S38">
-        <v>720.065307617188</v>
+        <v>715.791137695313</v>
       </c>
       <c r="T38">
-        <v>2.456787109375</v>
+        <v>-0.958984375</v>
       </c>
       <c r="U38">
-        <v>3.99322509765625</v>
+        <v>1.90118408203125</v>
       </c>
       <c r="V38">
-        <v>7.56854248046875</v>
+        <v>12.6798095703125</v>
       </c>
     </row>
     <row r="39" ht="19.5" customHeight="1">
-      <c r="A39" s="1">
-        <v>46211</v>
+      <c r="A39" s="2">
+        <v>46219</v>
       </c>
       <c r="B39">
-        <v>-4.7235107421875</v>
+        <v>-5.863037109375</v>
       </c>
       <c r="C39">
-        <v>-3.04364013671875</v>
+        <v>-2.36517333984375</v>
       </c>
       <c r="D39">
-        <v>-5.07476806640625</v>
+        <v>-3.09661865234375</v>
       </c>
       <c r="E39">
-        <v>704.950012207031</v>
+        <v>712.010009765625</v>
       </c>
       <c r="F39">
-        <v>712.259887695313</v>
+        <v>713.598999023438</v>
       </c>
       <c r="G39">
-        <v>700.909973144531</v>
+        <v>702.609985351563</v>
       </c>
       <c r="H39">
-        <v>711.440002441406</v>
+        <v>705.940002441406</v>
       </c>
       <c r="I39">
-        <v>715.620361328125</v>
+        <v>712.521850585938</v>
       </c>
       <c r="J39">
-        <v>704.994506835938</v>
+        <v>701.248962402344</v>
       </c>
       <c r="K39">
-        <v>35603100</v>
+        <v>39402000</v>
       </c>
       <c r="L39">
-        <v>-1.43523001670837</v>
+        <v>-1.98428201675415</v>
       </c>
       <c r="M39">
-        <v>55.0994873046875</v>
+        <v>50.0927925109863</v>
       </c>
       <c r="N39">
-        <v>-16.1432189941406</v>
+        <v>7.75767660140991</v>
       </c>
       <c r="O39" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P39">
-        <v>-15.6323156356812</v>
+        <v>-43.6580963134766</v>
       </c>
       <c r="Q39">
-        <v>712.987182617188</v>
+        <v>712.182556152344</v>
       </c>
       <c r="R39">
-        <v>717.214111328125</v>
+        <v>715.892822265625</v>
       </c>
       <c r="S39">
-        <v>719.531494140625</v>
+        <v>718.15576171875</v>
       </c>
       <c r="T39">
-        <v>3.3604736328125</v>
+        <v>-1.0771484375</v>
       </c>
       <c r="U39">
-        <v>4.08453369140625</v>
+        <v>-1.36102294921875</v>
       </c>
       <c r="V39">
-        <v>10.6258544921875</v>
+        <v>11.2728881835938</v>
       </c>
     </row>
     <row r="40" ht="19.5" customHeight="1">
-      <c r="A40" s="1">
-        <v>46210</v>
+      <c r="A40" s="2">
+        <v>46218</v>
       </c>
       <c r="B40">
-        <v>-7.9444580078125</v>
+        <v>-1.943359375</v>
       </c>
       <c r="C40">
-        <v>-0.99530029296875</v>
+        <v>0.40814208984375</v>
       </c>
       <c r="D40">
-        <v>-5.45904541015625</v>
+        <v>-0.0054931640625</v>
       </c>
       <c r="E40">
-        <v>714.169982910156</v>
+        <v>723.849975585938</v>
       </c>
       <c r="F40">
-        <v>716.349975585938</v>
+        <v>724.359985351563</v>
       </c>
       <c r="G40">
-        <v>704.900024414063</v>
+        <v>710.22998046875</v>
       </c>
       <c r="H40">
-        <v>709.429992675781</v>
+        <v>717.739990234375</v>
       </c>
       <c r="I40">
-        <v>714.261169433594</v>
+        <v>721.251037597656</v>
       </c>
       <c r="J40">
-        <v>704.237060546875</v>
+        <v>712.604736328125</v>
       </c>
       <c r="K40">
-        <v>42483000</v>
+        <v>32627500</v>
       </c>
       <c r="L40">
-        <v>-2.93475341796875</v>
+        <v>-1.41428053379059</v>
       </c>
       <c r="M40">
-        <v>65.706657409668</v>
+        <v>46.4865188598633</v>
       </c>
       <c r="N40">
-        <v>-6.48241281509399</v>
+        <v>-4.76508235931396</v>
       </c>
       <c r="O40" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P40">
-        <v>-38.1205101013184</v>
+        <v>-2.18429470062256</v>
       </c>
       <c r="Q40">
-        <v>715.312561035156</v>
+        <v>717.8037109375</v>
       </c>
       <c r="R40">
-        <v>718.993896484375</v>
+        <v>718.531005859375</v>
       </c>
       <c r="S40">
-        <v>720.435485839844</v>
+        <v>719.552307128906</v>
       </c>
       <c r="T40">
-        <v>-2.08880615234375</v>
+        <v>-3.10894775390625</v>
       </c>
       <c r="U40">
-        <v>-0.6629638671875</v>
+        <v>2.374755859375</v>
       </c>
       <c r="V40">
-        <v>10.0241088867188</v>
+        <v>8.64630126953125</v>
       </c>
     </row>
     <row r="41" ht="19.5" customHeight="1">
-      <c r="A41" s="1">
-        <v>46209</v>
+      <c r="A41" s="2">
+        <v>46217</v>
       </c>
       <c r="B41">
-        <v>-2.8165283203125</v>
+        <v>0.21160888671875</v>
       </c>
       <c r="C41">
-        <v>0.947509765625</v>
+        <v>-1.59527587890625</v>
       </c>
       <c r="D41">
-        <v>-2.495361328125</v>
+        <v>0.46612548828125</v>
       </c>
       <c r="E41">
-        <v>719.929992675781</v>
+        <v>720.219970703125</v>
       </c>
       <c r="F41">
-        <v>726.080017089844</v>
+        <v>722.289978027344</v>
       </c>
       <c r="G41">
-        <v>718.450012207031</v>
+        <v>714.340026855469</v>
       </c>
       <c r="H41">
-        <v>722.820007324219</v>
+        <v>719.690002441406</v>
       </c>
       <c r="I41">
-        <v>729.223693847656</v>
+        <v>723.544555664063</v>
       </c>
       <c r="J41">
-        <v>718.437683105469</v>
+        <v>716.334533691406</v>
       </c>
       <c r="K41">
-        <v>30220400</v>
+        <v>29448100</v>
       </c>
       <c r="L41">
-        <v>-2.4647536277771</v>
+        <v>-0.94570779800415</v>
       </c>
       <c r="M41">
-        <v>70.2612838745117</v>
+        <v>48.8124732971191</v>
       </c>
       <c r="N41">
-        <v>3.65661525726318</v>
+        <v>-5.16571569442749</v>
       </c>
       <c r="O41" t="s">
         <v>1</v>
       </c>
       <c r="P41">
-        <v>18.3796253204346</v>
+        <v>5.93372297286987</v>
       </c>
       <c r="Q41">
-        <v>721.317932128906</v>
+        <v>718.3955078125</v>
       </c>
       <c r="R41">
-        <v>721.685180664063</v>
+        <v>718.438903808594</v>
       </c>
       <c r="S41">
-        <v>721.850463867188</v>
+        <v>719.708923339844</v>
       </c>
       <c r="T41">
-        <v>3.1436767578125</v>
+        <v>1.25457763671875</v>
       </c>
       <c r="U41">
-        <v>-0.0123291015625</v>
+        <v>1.9945068359375</v>
       </c>
       <c r="V41">
-        <v>10.7860107421875</v>
+        <v>7.21002197265625</v>
       </c>
     </row>
     <row r="42" ht="19.5" customHeight="1">
-      <c r="A42" s="1">
-        <v>46205</v>
+      <c r="A42" s="2">
+        <v>46216</v>
       </c>
       <c r="B42">
-        <v>-3.747802734375</v>
+        <v>-0.3555908203125</v>
       </c>
       <c r="C42">
-        <v>-2.68170166015625</v>
+        <v>-3.0672607421875</v>
       </c>
       <c r="D42">
-        <v>-3.40606689453125</v>
+        <v>-1.38330078125</v>
       </c>
       <c r="E42">
-        <v>725.580017089844</v>
+        <v>717.719970703125</v>
       </c>
       <c r="F42">
-        <v>730.830017089844</v>
+        <v>718.739990234375</v>
       </c>
       <c r="G42">
-        <v>707.559997558594</v>
+        <v>710.080017089844</v>
       </c>
       <c r="H42">
-        <v>712.599975585938</v>
+        <v>711.739990234375</v>
       </c>
       <c r="I42">
-        <v>718.628479003906</v>
+        <v>717.577209472656</v>
       </c>
       <c r="J42">
-        <v>705.427856445313</v>
+        <v>707.793212890625</v>
       </c>
       <c r="K42">
-        <v>51086000</v>
+        <v>36552300</v>
       </c>
       <c r="L42">
-        <v>-2.74999117851257</v>
+        <v>-0.0714227557182312</v>
       </c>
       <c r="M42">
-        <v>67.7827301025391</v>
+        <v>51.4713363647461</v>
       </c>
       <c r="N42">
-        <v>14.6252498626709</v>
+        <v>4.72496747970581</v>
       </c>
       <c r="O42" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P42">
-        <v>-52.3691177368164</v>
+        <v>-42.1362648010254</v>
       </c>
       <c r="Q42">
-        <v>719.125122070313</v>
+        <v>716.920593261719</v>
       </c>
       <c r="R42">
-        <v>720.899353027344</v>
+        <v>718.116577148438</v>
       </c>
       <c r="S42">
-        <v>721.46142578125</v>
+        <v>719.618469238281</v>
       </c>
       <c r="T42">
-        <v>-12.2015380859375</v>
+        <v>-1.16278076171875</v>
       </c>
       <c r="U42">
-        <v>-2.13214111328125</v>
+        <v>-2.28680419921875</v>
       </c>
       <c r="V42">
-        <v>13.2006225585938</v>
+        <v>9.78399658203125</v>
       </c>
     </row>
     <row r="43" ht="19.5" customHeight="1">
-      <c r="A43" s="1">
-        <v>46204</v>
+      <c r="A43" s="2">
+        <v>46213</v>
       </c>
       <c r="B43">
-        <v>5.48199462890625</v>
+        <v>4.54119873046875</v>
       </c>
       <c r="C43">
-        <v>1.29547119140625</v>
+        <v>1.09893798828125</v>
       </c>
       <c r="D43">
-        <v>1.181640625</v>
+        <v>-0.62530517578125</v>
       </c>
       <c r="E43">
-        <v>729.190002441406</v>
+        <v>720.700012207031</v>
       </c>
       <c r="F43">
-        <v>731.919982910156</v>
+        <v>726.390014648438</v>
       </c>
       <c r="G43">
-        <v>724.599975585938</v>
+        <v>717</v>
       </c>
       <c r="H43">
-        <v>725.169982910156</v>
+        <v>725.510009765625</v>
       </c>
       <c r="I43">
-        <v>731.202941894531</v>
+        <v>728.048034667969</v>
       </c>
       <c r="J43">
-        <v>721.92822265625</v>
+        <v>721.283996582031</v>
       </c>
       <c r="K43">
-        <v>40803700</v>
+        <v>26415900</v>
       </c>
       <c r="L43">
-        <v>-1.9528489112854</v>
+        <v>-0.166184201836586</v>
       </c>
       <c r="M43">
-        <v>59.134204864502</v>
+        <v>49.1490592956543</v>
       </c>
       <c r="N43">
-        <v>25.8970050811768</v>
+        <v>-9.55446624755859</v>
       </c>
       <c r="O43" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="P43">
-        <v>-6.59338569641113</v>
+        <v>29.1831836700439</v>
       </c>
       <c r="Q43">
-        <v>726.038452148438</v>
+        <v>721.479248046875</v>
       </c>
       <c r="R43">
-        <v>723.370727539063</v>
+        <v>719.98193359375</v>
       </c>
       <c r="S43">
-        <v>722.493774414063</v>
+        <v>720.620422363281</v>
       </c>
       <c r="T43">
-        <v>-0.717041015625</v>
+        <v>1.65802001953125</v>
       </c>
       <c r="U43">
-        <v>-2.6717529296875</v>
+        <v>4.28399658203125</v>
       </c>
       <c r="V43">
-        <v>9.27471923828125</v>
+        <v>6.7640380859375</v>
       </c>
     </row>
     <row r="44" ht="19.5" customHeight="1">
-      <c r="A44" s="1">
-        <v>46203</v>
+      <c r="A44" s="2">
+        <v>46212</v>
       </c>
       <c r="B44">
-        <v>10.5760498046875</v>
+        <v>3.296630859375</v>
       </c>
       <c r="C44">
-        <v>1.1090087890625</v>
+        <v>-0.72021484375</v>
       </c>
       <c r="D44">
-        <v>2.15655517578125</v>
+        <v>-2.30474853515625</v>
       </c>
       <c r="E44">
-        <v>724.179992675781</v>
+        <v>718.330017089844</v>
       </c>
       <c r="F44">
-        <v>737.619995117188</v>
+        <v>724.22998046875</v>
       </c>
       <c r="G44">
-        <v>723.909973144531</v>
+        <v>715.125</v>
       </c>
       <c r="H44">
-        <v>736.400024414063</v>
+        <v>723.280029296875</v>
       </c>
       <c r="I44">
-        <v>740.130432128906</v>
+        <v>726.686767578125</v>
       </c>
       <c r="J44">
-        <v>729.166198730469</v>
+        <v>719.118225097656</v>
       </c>
       <c r="K44">
-        <v>42121800</v>
+        <v>33654700</v>
       </c>
       <c r="L44">
-        <v>-1.489990234375</v>
+        <v>-1.11665856838226</v>
       </c>
       <c r="M44">
-        <v>46.9703025817871</v>
+        <v>54.3410568237305</v>
       </c>
       <c r="N44">
-        <v>-18.5084857940674</v>
+        <v>-1.37647461891174</v>
       </c>
       <c r="O44" t="s">
         <v>1</v>
       </c>
       <c r="P44">
-        <v>57.9281425476074</v>
+        <v>56.2780990600586</v>
       </c>
       <c r="Q44">
-        <v>725.990234375</v>
+        <v>718.006164550781</v>
       </c>
       <c r="R44">
-        <v>723.10791015625</v>
+        <v>718.503051757813</v>
       </c>
       <c r="S44">
-        <v>722.2724609375</v>
+        <v>720.065307617188</v>
       </c>
       <c r="T44">
-        <v>2.51043701171875</v>
+        <v>2.456787109375</v>
       </c>
       <c r="U44">
-        <v>5.2562255859375</v>
+        <v>3.99322509765625</v>
       </c>
       <c r="V44">
-        <v>10.9642333984375</v>
+        <v>7.56854248046875</v>
       </c>
     </row>
     <row r="45" ht="19.5" customHeight="1">
-      <c r="A45" s="1">
-        <v>46202</v>
+      <c r="A45" s="2">
+        <v>46211</v>
       </c>
       <c r="B45">
-        <v>3.40582275390625</v>
+        <v>-4.7235107421875</v>
       </c>
       <c r="C45">
-        <v>-7.25604248046875</v>
+        <v>-3.04364013671875</v>
       </c>
       <c r="D45">
-        <v>-1.9508056640625</v>
+        <v>-5.07476806640625</v>
       </c>
       <c r="E45">
-        <v>713.989990234375</v>
+        <v>704.950012207031</v>
       </c>
       <c r="F45">
-        <v>724.580017089844</v>
+        <v>712.259887695313</v>
       </c>
       <c r="G45">
-        <v>705.171997070313</v>
+        <v>700.909973144531</v>
       </c>
       <c r="H45">
-        <v>724.080017089844</v>
+        <v>711.440002441406</v>
       </c>
       <c r="I45">
-        <v>725.809997558594</v>
+        <v>715.620361328125</v>
       </c>
       <c r="J45">
-        <v>714.771484375</v>
+        <v>704.994506835938</v>
       </c>
       <c r="K45">
-        <v>44939000</v>
+        <v>35603100</v>
       </c>
       <c r="L45">
-        <v>-2.04951691627502</v>
+        <v>-1.43523001670837</v>
       </c>
       <c r="M45">
-        <v>57.6382751464844</v>
+        <v>55.0994873046875</v>
       </c>
       <c r="N45">
-        <v>-16.8400115966797</v>
+        <v>-16.1432189941406</v>
       </c>
       <c r="O45" t="s">
+        <v>23</v>
+      </c>
+      <c r="P45">
+        <v>-15.6323156356812</v>
+      </c>
+      <c r="Q45">
+        <v>712.987182617188</v>
+      </c>
+      <c r="R45">
+        <v>717.214111328125</v>
+      </c>
+      <c r="S45">
+        <v>719.531494140625</v>
+      </c>
+      <c r="T45">
+        <v>3.3604736328125</v>
+      </c>
+      <c r="U45">
+        <v>4.08453369140625</v>
+      </c>
+      <c r="V45">
+        <v>10.6258544921875</v>
+      </c>
+    </row>
+    <row r="46" ht="19.5" customHeight="1">
+      <c r="A46" s="2">
+        <v>46210</v>
+      </c>
+      <c r="B46">
+        <v>-7.9444580078125</v>
+      </c>
+      <c r="C46">
+        <v>-0.99530029296875</v>
+      </c>
+      <c r="D46">
+        <v>-5.45904541015625</v>
+      </c>
+      <c r="E46">
+        <v>714.169982910156</v>
+      </c>
+      <c r="F46">
+        <v>716.349975585938</v>
+      </c>
+      <c r="G46">
+        <v>704.900024414063</v>
+      </c>
+      <c r="H46">
+        <v>709.429992675781</v>
+      </c>
+      <c r="I46">
+        <v>714.261169433594</v>
+      </c>
+      <c r="J46">
+        <v>704.237060546875</v>
+      </c>
+      <c r="K46">
+        <v>42483000</v>
+      </c>
+      <c r="L46">
+        <v>-2.93475341796875</v>
+      </c>
+      <c r="M46">
+        <v>65.706657409668</v>
+      </c>
+      <c r="N46">
+        <v>-6.48241281509399</v>
+      </c>
+      <c r="O46" t="s">
+        <v>23</v>
+      </c>
+      <c r="P46">
+        <v>-38.1205101013184</v>
+      </c>
+      <c r="Q46">
+        <v>715.312561035156</v>
+      </c>
+      <c r="R46">
+        <v>718.993896484375</v>
+      </c>
+      <c r="S46">
+        <v>720.435485839844</v>
+      </c>
+      <c r="T46">
+        <v>-2.08880615234375</v>
+      </c>
+      <c r="U46">
+        <v>-0.6629638671875</v>
+      </c>
+      <c r="V46">
+        <v>10.0241088867188</v>
+      </c>
+    </row>
+    <row r="47" ht="19.5" customHeight="1">
+      <c r="A47" s="2">
+        <v>46209</v>
+      </c>
+      <c r="B47">
+        <v>-2.8165283203125</v>
+      </c>
+      <c r="C47">
+        <v>0.947509765625</v>
+      </c>
+      <c r="D47">
+        <v>-2.495361328125</v>
+      </c>
+      <c r="E47">
+        <v>719.929992675781</v>
+      </c>
+      <c r="F47">
+        <v>726.080017089844</v>
+      </c>
+      <c r="G47">
+        <v>718.450012207031</v>
+      </c>
+      <c r="H47">
+        <v>722.820007324219</v>
+      </c>
+      <c r="I47">
+        <v>729.223693847656</v>
+      </c>
+      <c r="J47">
+        <v>718.437683105469</v>
+      </c>
+      <c r="K47">
+        <v>30220400</v>
+      </c>
+      <c r="L47">
+        <v>-2.4647536277771</v>
+      </c>
+      <c r="M47">
+        <v>70.2612838745117</v>
+      </c>
+      <c r="N47">
+        <v>3.65661525726318</v>
+      </c>
+      <c r="O47" t="s">
         <v>1</v>
       </c>
-      <c r="P45">
-        <v>20.9863204956055</v>
-      </c>
-      <c r="Q45">
-        <v>716.725952148438</v>
-      </c>
-      <c r="R45">
-        <v>719.314147949219</v>
-      </c>
-      <c r="S45">
-        <v>720.439880371094</v>
-      </c>
-      <c r="T45">
-        <v>1.22998046875</v>
-      </c>
-      <c r="U45">
-        <v>9.5994873046875</v>
-      </c>
-      <c r="V45">
-        <v>11.0385131835938</v>
+      <c r="P47">
+        <v>18.3796253204346</v>
+      </c>
+      <c r="Q47">
+        <v>721.317932128906</v>
+      </c>
+      <c r="R47">
+        <v>721.685180664063</v>
+      </c>
+      <c r="S47">
+        <v>721.850463867188</v>
+      </c>
+      <c r="T47">
+        <v>3.1436767578125</v>
+      </c>
+      <c r="U47">
+        <v>-0.0123291015625</v>
+      </c>
+      <c r="V47">
+        <v>10.7860107421875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>